<commit_message>
Add interactive economics scenario lab
Add a guided model-sensitivity exercise with formula-driven scenarios, identification warnings, and updated portfolio instructions.
</commit_message>
<xml_diff>
--- a/Scam_Geography_Interactive_Economics_Project.xlsx
+++ b/Scam_Geography_Interactive_Economics_Project.xlsx
@@ -2,16 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rab1cdb4281114e14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Re497712f04cf4f88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Data" sheetId="3" r:id="Ra7e63c07b3aa48e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression" sheetId="4" r:id="R85eae07a8bb24653"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Notes" sheetId="5" r:id="Rfdd73c6033d34741"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart Data" sheetId="6" r:id="R4a52f703274d42f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Dashboard" sheetId="7" r:id="Rde7c556f03c443a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Data" sheetId="8" r:id="Racaa2c8238de4715"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Models" sheetId="9" r:id="R119b9d6a1cfa4e6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interactive Econ Lab" sheetId="10" r:id="Rca940365b08846ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R7b3bcbd1117e4243"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rcbe497e5469e47d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Data" sheetId="3" r:id="R2ea294a6ed274f6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression" sheetId="4" r:id="Rd0996dc604a1444a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Notes" sheetId="5" r:id="R47a48af8072a4974"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart Data" sheetId="6" r:id="R1123ad6d48844da4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Dashboard" sheetId="7" r:id="Re9a6b261708b4dfd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Data" sheetId="8" r:id="R84bd9eaaf3344eb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Models" sheetId="9" r:id="R3201faeecf114164"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interactive Econ Lab" sheetId="10" r:id="Rd59d8974eca346bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Lab" sheetId="11" r:id="R7d4d4114a8224a4d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,7 +23,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="12">
+  <x:numFmts count="13">
     <x:numFmt numFmtId="200" formatCode="0%"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
     <x:numFmt numFmtId="202" formatCode="0"/>
@@ -35,8 +36,9 @@
     <x:numFmt numFmtId="209" formatCode="0.0000"/>
     <x:numFmt numFmtId="210" formatCode="#,##0.00"/>
     <x:numFmt numFmtId="211" formatCode="+0%;-0%;0%"/>
+    <x:numFmt numFmtId="212" formatCode="+0.0%;-0.0%;0.0%"/>
   </x:numFmts>
-  <x:fonts count="20">
+  <x:fonts count="21">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -149,6 +151,12 @@
       <x:color rgb="FF17324D"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FF17324D"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
   <x:fills count="13">
     <x:fill>
@@ -213,7 +221,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="34">
+  <x:borders count="36">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -431,11 +439,33 @@
         <x:color rgb="FFD99B2B"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFC5D3DC"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFC5D3DC"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFC5D3DC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFC5D3DC"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFC5D3DC"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFC5D3DC"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="353">
+  <x:cellXfs count="365">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1155,6 +1185,28 @@
     <x:xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="19" fillId="12" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="20" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="20" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="20" fillId="6" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="20" fillId="6" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="20" fillId="6" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="20" fillId="6" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="212" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1664,6 +1716,144 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/drawings/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:t>How model choice changes the scenario</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Baseline</c:v>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Scenario Lab'!$A$12:$A$14</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Scenario Lab'!$C$12:$C$14</c:f>
+              <c:numCache>
+                <c:formatCode>$0</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Scenario</c:v>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Scenario Lab'!$A$12:$A$14</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Scenario Lab'!$D$12:$D$14</c:f>
+              <c:numCache>
+                <c:formatCode>$0</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="48672768"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="$0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
@@ -1690,7 +1880,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc32b60024eaf4879"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3b04e7e3992449ce"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1720,7 +1910,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd0107fc84ce1420e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4f97da1c400a4646"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1755,7 +1945,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R13fdf32d4f484896"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6062a277b44c445f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1790,7 +1980,42 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4730103cfd99454c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re34d5bea8cef4c8a"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R31146cf556f54f5e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2187,9 +2412,9 @@
       <x:c r="I7" s="31"/>
       <x:c r="K7" s="57" t="str">
         <x:v>1. Open Interactive Econ Lab
-2. Change the four yellow controls
-3. Compare exposure vs. severity
-4. Read the model verdict
+2. Compare states and outcomes
+3. Open Scenario Lab
+4. Test an income-change scenario
 5. Check Sources &amp; Notes</x:v>
       </x:c>
       <x:c r="L7" s="58"/>
@@ -3038,7 +3263,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b7516cdcdd04ac4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf59289ecaef47d3"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -3051,6 +3276,490 @@
             </x14:dataBar>
           </x14:cfRule>
           <xm:sqref>D11:D14</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </x:ext>
+  </x:extLst>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="324" t="str">
+        <x:v>SCENARIO LAB — WHAT WOULD THE MODELS IMPLY?</x:v>
+      </x:c>
+      <x:c r="B1" s="324"/>
+      <x:c r="C1" s="324"/>
+      <x:c r="D1" s="324"/>
+      <x:c r="E1" s="324"/>
+      <x:c r="F1" s="324"/>
+      <x:c r="G1" s="324"/>
+      <x:c r="H1" s="324"/>
+      <x:c r="I1" s="324"/>
+      <x:c r="J1" s="324"/>
+      <x:c r="K1" s="324"/>
+      <x:c r="L1" s="324"/>
+      <x:c r="M1" s="324"/>
+      <x:c r="N1" s="324"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="324"/>
+      <x:c r="B2" s="324"/>
+      <x:c r="C2" s="324"/>
+      <x:c r="D2" s="324"/>
+      <x:c r="E2" s="324"/>
+      <x:c r="F2" s="324"/>
+      <x:c r="G2" s="324"/>
+      <x:c r="H2" s="324"/>
+      <x:c r="I2" s="324"/>
+      <x:c r="J2" s="324"/>
+      <x:c r="K2" s="324"/>
+      <x:c r="L2" s="324"/>
+      <x:c r="M2" s="324"/>
+      <x:c r="N2" s="324"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="354" t="str">
+        <x:v>Choose a state, year, and hypothetical income change. The workbook translates each estimated elasticity into a model-implied loss-per-person scenario.</x:v>
+      </x:c>
+      <x:c r="B3" s="354"/>
+      <x:c r="C3" s="354"/>
+      <x:c r="D3" s="354"/>
+      <x:c r="E3" s="354"/>
+      <x:c r="F3" s="354"/>
+      <x:c r="G3" s="354"/>
+      <x:c r="H3" s="354"/>
+      <x:c r="I3" s="354"/>
+      <x:c r="J3" s="354"/>
+      <x:c r="K3" s="354"/>
+      <x:c r="L3" s="354"/>
+      <x:c r="M3" s="354"/>
+      <x:c r="N3" s="354"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="68" t="str">
+        <x:v>State</x:v>
+      </x:c>
+      <x:c r="B5" s="68"/>
+      <x:c r="C5" s="68"/>
+      <x:c r="D5" s="68" t="str">
+        <x:v>Year</x:v>
+      </x:c>
+      <x:c r="E5" s="68"/>
+      <x:c r="F5" s="68"/>
+      <x:c r="G5" s="68" t="str">
+        <x:v>Income change</x:v>
+      </x:c>
+      <x:c r="H5" s="68"/>
+      <x:c r="I5" s="68"/>
+      <x:c r="K5" s="37" t="str">
+        <x:v>BASELINE</x:v>
+      </x:c>
+      <x:c r="L5" s="37"/>
+      <x:c r="M5" s="37"/>
+      <x:c r="N5" s="37"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="339" t="str">
+        <x:v>North Carolina</x:v>
+      </x:c>
+      <x:c r="B6" s="340"/>
+      <x:c r="C6" s="341"/>
+      <x:c r="D6" s="339" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="E6" s="340"/>
+      <x:c r="F6" s="341"/>
+      <x:c r="G6" s="355" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="H6" s="340"/>
+      <x:c r="I6" s="341"/>
+      <x:c r="K6" s="316" t="str">
+        <x:v>Median income</x:v>
+      </x:c>
+      <x:c r="L6" s="316" t="str">
+        <x:v>Loss / person</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="342"/>
+      <x:c r="B7" s="343"/>
+      <x:c r="C7" s="344"/>
+      <x:c r="D7" s="342"/>
+      <x:c r="E7" s="343"/>
+      <x:c r="F7" s="344"/>
+      <x:c r="G7" s="342"/>
+      <x:c r="H7" s="343"/>
+      <x:c r="I7" s="344"/>
+      <x:c r="K7" s="362" t="n">
+        <x:f>SUMIFS('Panel Data'!$F$2:$F$205,'Panel Data'!$A$2:$A$205,$D$6,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
+        <x:v>73958</x:v>
+      </x:c>
+      <x:c r="L7" s="363" t="n">
+        <x:f>SUMIFS('Panel Data'!$L$2:$L$205,'Panel Data'!$A$2:$A$205,$D$6,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
+        <x:v>39.06941683269926</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="36" t="str">
+        <x:v>MODEL-IMPLIED LOSS PER PERSON</x:v>
+      </x:c>
+      <x:c r="B10" s="36"/>
+      <x:c r="C10" s="36"/>
+      <x:c r="D10" s="36"/>
+      <x:c r="E10" s="36"/>
+      <x:c r="F10" s="36"/>
+      <x:c r="G10" s="36"/>
+      <x:c r="H10" s="36"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="316" t="str">
+        <x:v>Evidence lens</x:v>
+      </x:c>
+      <x:c r="B11" s="316" t="str">
+        <x:v>Income elasticity</x:v>
+      </x:c>
+      <x:c r="C11" s="316" t="str">
+        <x:v>Baseline</x:v>
+      </x:c>
+      <x:c r="D11" s="316" t="str">
+        <x:v>Scenario</x:v>
+      </x:c>
+      <x:c r="E11" s="316" t="str">
+        <x:v>Change</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>Pooled + year effects</x:v>
+      </x:c>
+      <x:c r="B12" s="263" t="n">
+        <x:v>1.552</x:v>
+      </x:c>
+      <x:c r="C12" s="225" t="n">
+        <x:f>$L$7</x:f>
+        <x:v>39.06941683269926</x:v>
+      </x:c>
+      <x:c r="D12" s="225" t="n">
+        <x:f>C12*(1+$G$6)^B12</x:f>
+        <x:v>45.297932070756154</x:v>
+      </x:c>
+      <x:c r="E12" s="364" t="n">
+        <x:f>D12/C12-1</x:f>
+        <x:v>0.15942176113680606</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>State + year fixed effects</x:v>
+      </x:c>
+      <x:c r="B13" s="263" t="n">
+        <x:v>2.188</x:v>
+      </x:c>
+      <x:c r="C13" s="225" t="n">
+        <x:f>$L$7</x:f>
+        <x:v>39.06941683269926</x:v>
+      </x:c>
+      <x:c r="D13" s="225" t="n">
+        <x:f>C13*(1+$G$6)^B13</x:f>
+        <x:v>48.12869920014451</x:v>
+      </x:c>
+      <x:c r="E13" s="364" t="n">
+        <x:f>D13/C13-1</x:f>
+        <x:v>0.23187657000969253</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>Exclude D.C. robustness</x:v>
+      </x:c>
+      <x:c r="B14" s="263" t="n">
+        <x:v>0.887</x:v>
+      </x:c>
+      <x:c r="C14" s="225" t="n">
+        <x:f>$L$7</x:f>
+        <x:v>39.06941683269926</x:v>
+      </x:c>
+      <x:c r="D14" s="225" t="n">
+        <x:f>C14*(1+$G$6)^B14</x:f>
+        <x:v>42.51598454771643</x:v>
+      </x:c>
+      <x:c r="E14" s="364" t="n">
+        <x:f>D14/C14-1</x:f>
+        <x:v>0.0882165129255923</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="112" t="str">
+        <x:v>HOW TO READ IT</x:v>
+      </x:c>
+      <x:c r="B17" s="112"/>
+      <x:c r="C17" s="112"/>
+      <x:c r="D17" s="112"/>
+      <x:c r="E17" s="112"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="160" t="str">
+        <x:v>Elasticity translates percentage changes into model-implied outcome changes. For example, an elasticity of 1.55 means a 10% income difference is associated with roughly a 15.9% difference in loss per person using the exact power formula.
+Compare the three rows. Their spread is model uncertainty—not three competing facts.</x:v>
+      </x:c>
+      <x:c r="B18" s="161"/>
+      <x:c r="C18" s="161"/>
+      <x:c r="D18" s="161"/>
+      <x:c r="E18" s="162"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="163"/>
+      <x:c r="B19" s="164"/>
+      <x:c r="C19" s="164"/>
+      <x:c r="D19" s="164"/>
+      <x:c r="E19" s="165"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="163"/>
+      <x:c r="B20" s="164"/>
+      <x:c r="C20" s="164"/>
+      <x:c r="D20" s="164"/>
+      <x:c r="E20" s="165"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="163"/>
+      <x:c r="B21" s="164"/>
+      <x:c r="C21" s="164"/>
+      <x:c r="D21" s="164"/>
+      <x:c r="E21" s="165"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="163"/>
+      <x:c r="B22" s="164"/>
+      <x:c r="C22" s="164"/>
+      <x:c r="D22" s="164"/>
+      <x:c r="E22" s="165"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="163"/>
+      <x:c r="B23" s="164"/>
+      <x:c r="C23" s="164"/>
+      <x:c r="D23" s="164"/>
+      <x:c r="E23" s="165"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="166"/>
+      <x:c r="B24" s="167"/>
+      <x:c r="C24" s="167"/>
+      <x:c r="D24" s="167"/>
+      <x:c r="E24" s="168"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="349" t="str">
+        <x:v>IMPORTANT: THIS IS NOT A CAUSAL FORECAST
+The elasticities describe associations in state-level data. Changing income alone would not mechanically cause the displayed change in fraud loss. Reporting behavior, target value, internet exposure, enforcement, and omitted state characteristics may all contribute. Use this lab to study sensitivity and identification—not to predict policy effects.</x:v>
+      </x:c>
+      <x:c r="B27" s="349"/>
+      <x:c r="C27" s="349"/>
+      <x:c r="D27" s="349"/>
+      <x:c r="E27" s="349"/>
+      <x:c r="F27" s="349"/>
+      <x:c r="G27" s="349"/>
+      <x:c r="H27" s="349"/>
+      <x:c r="I27" s="349"/>
+      <x:c r="J27" s="349"/>
+      <x:c r="K27" s="349"/>
+      <x:c r="L27" s="349"/>
+      <x:c r="M27" s="349"/>
+      <x:c r="N27" s="349"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="349"/>
+      <x:c r="B28" s="349"/>
+      <x:c r="C28" s="349"/>
+      <x:c r="D28" s="349"/>
+      <x:c r="E28" s="349"/>
+      <x:c r="F28" s="349"/>
+      <x:c r="G28" s="349"/>
+      <x:c r="H28" s="349"/>
+      <x:c r="I28" s="349"/>
+      <x:c r="J28" s="349"/>
+      <x:c r="K28" s="349"/>
+      <x:c r="L28" s="349"/>
+      <x:c r="M28" s="349"/>
+      <x:c r="N28" s="349"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="349"/>
+      <x:c r="B29" s="349"/>
+      <x:c r="C29" s="349"/>
+      <x:c r="D29" s="349"/>
+      <x:c r="E29" s="349"/>
+      <x:c r="F29" s="349"/>
+      <x:c r="G29" s="349"/>
+      <x:c r="H29" s="349"/>
+      <x:c r="I29" s="349"/>
+      <x:c r="J29" s="349"/>
+      <x:c r="K29" s="349"/>
+      <x:c r="L29" s="349"/>
+      <x:c r="M29" s="349"/>
+      <x:c r="N29" s="349"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="349"/>
+      <x:c r="B30" s="349"/>
+      <x:c r="C30" s="349"/>
+      <x:c r="D30" s="349"/>
+      <x:c r="E30" s="349"/>
+      <x:c r="F30" s="349"/>
+      <x:c r="G30" s="349"/>
+      <x:c r="H30" s="349"/>
+      <x:c r="I30" s="349"/>
+      <x:c r="J30" s="349"/>
+      <x:c r="K30" s="349"/>
+      <x:c r="L30" s="349"/>
+      <x:c r="M30" s="349"/>
+      <x:c r="N30" s="349"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="349"/>
+      <x:c r="B31" s="349"/>
+      <x:c r="C31" s="349"/>
+      <x:c r="D31" s="349"/>
+      <x:c r="E31" s="349"/>
+      <x:c r="F31" s="349"/>
+      <x:c r="G31" s="349"/>
+      <x:c r="H31" s="349"/>
+      <x:c r="I31" s="349"/>
+      <x:c r="J31" s="349"/>
+      <x:c r="K31" s="349"/>
+      <x:c r="L31" s="349"/>
+      <x:c r="M31" s="349"/>
+      <x:c r="N31" s="349"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="354" t="str">
+        <x:v>CHALLENGE: Set income change to +10%. Which specification produces the smallest implied change? Why might the fixed-effects estimate be less precise even though its point estimate is larger?</x:v>
+      </x:c>
+      <x:c r="B33" s="354"/>
+      <x:c r="C33" s="354"/>
+      <x:c r="D33" s="354"/>
+      <x:c r="E33" s="354"/>
+      <x:c r="F33" s="354"/>
+      <x:c r="G33" s="354"/>
+      <x:c r="H33" s="354"/>
+      <x:c r="I33" s="354"/>
+      <x:c r="J33" s="354"/>
+      <x:c r="K33" s="354"/>
+      <x:c r="L33" s="354"/>
+      <x:c r="M33" s="354"/>
+      <x:c r="N33" s="354"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="354"/>
+      <x:c r="B34" s="354"/>
+      <x:c r="C34" s="354"/>
+      <x:c r="D34" s="354"/>
+      <x:c r="E34" s="354"/>
+      <x:c r="F34" s="354"/>
+      <x:c r="G34" s="354"/>
+      <x:c r="H34" s="354"/>
+      <x:c r="I34" s="354"/>
+      <x:c r="J34" s="354"/>
+      <x:c r="K34" s="354"/>
+      <x:c r="L34" s="354"/>
+      <x:c r="M34" s="354"/>
+      <x:c r="N34" s="354"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="354"/>
+      <x:c r="B35" s="354"/>
+      <x:c r="C35" s="354"/>
+      <x:c r="D35" s="354"/>
+      <x:c r="E35" s="354"/>
+      <x:c r="F35" s="354"/>
+      <x:c r="G35" s="354"/>
+      <x:c r="H35" s="354"/>
+      <x:c r="I35" s="354"/>
+      <x:c r="J35" s="354"/>
+      <x:c r="K35" s="354"/>
+      <x:c r="L35" s="354"/>
+      <x:c r="M35" s="354"/>
+      <x:c r="N35" s="354"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:N2"/>
+    <x:mergeCell ref="A3:N3"/>
+    <x:mergeCell ref="A5:C5"/>
+    <x:mergeCell ref="D5:F5"/>
+    <x:mergeCell ref="G5:I5"/>
+    <x:mergeCell ref="A6:C7"/>
+    <x:mergeCell ref="D6:F7"/>
+    <x:mergeCell ref="G6:I7"/>
+    <x:mergeCell ref="K5:N5"/>
+    <x:mergeCell ref="A10:H10"/>
+    <x:mergeCell ref="A17:E17"/>
+    <x:mergeCell ref="A18:E24"/>
+    <x:mergeCell ref="A27:N31"/>
+    <x:mergeCell ref="A33:N35"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="E12:E14">
+    <x:cfRule type="dataBar" priority="1">
+      <x:dataBar>
+        <x:cfvo type="min"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FF2A9D8F"/>
+      </x:dataBar>
+      <x:extLst>
+        <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{CB2FE225-2CFD-8AD7-C75C-B7D01DF273F4}</x14:id>
+        </x:ext>
+      </x:extLst>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="3">
+    <x:dataValidation type="list" sqref="A6">
+      <x:formula1>'Chart Data'!$A$2:$A$52</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D6">
+      <x:formula1>"2022,2023,2024,2025"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="between" sqref="G6">
+      <x:formula1>-0.5</x:formula1>
+      <x:formula2>1</x:formula2>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf55c8bf5eebd4686"/>
+  <x:extLst>
+    <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting>
+          <x14:cfRule type="dataBar" priority="1" id="{CB2FE225-2CFD-8AD7-C75C-B7D01DF273F4}">
+            <x14:dataBar gradient="1">
+              <x14:cfvo type="min"/>
+              <x14:cfvo type="max"/>
+              <x14:fillColor rgb="FF2A9D8F"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E12:E14</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </x:ext>
@@ -3466,7 +4175,7 @@
     <x:mergeCell ref="A40:N42"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc04ae5c174424614"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc07663cb080845fa"/>
 </x:worksheet>
 </file>
 
@@ -6570,7 +7279,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1bea02cc0114a1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba01d9a565d24c64"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6987,7 +7696,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dfdc67bdcdd40c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7baa045060714aa2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8265,7 +8974,7 @@
     <x:mergeCell ref="A30:N33"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R132945cdf8c747bb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra29926aca0334437"/>
 </x:worksheet>
 </file>
 
@@ -18540,7 +19249,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f9ef2228b084441"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d9aa9fb2b4a4a1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19105,7 +19814,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d734bb78f88443e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68efd47c9c144a3b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add interactive state economics scorecard
Add formula-driven percentiles, exposure-severity quadrants, state rankings, and an interactive four-year profile.
</commit_message>
<xml_diff>
--- a/Scam_Geography_Interactive_Economics_Project.xlsx
+++ b/Scam_Geography_Interactive_Economics_Project.xlsx
@@ -2,17 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R7b3bcbd1117e4243"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rcbe497e5469e47d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Data" sheetId="3" r:id="R2ea294a6ed274f6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression" sheetId="4" r:id="Rd0996dc604a1444a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Notes" sheetId="5" r:id="R47a48af8072a4974"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart Data" sheetId="6" r:id="R1123ad6d48844da4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Dashboard" sheetId="7" r:id="Re9a6b261708b4dfd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Data" sheetId="8" r:id="R84bd9eaaf3344eb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Models" sheetId="9" r:id="R3201faeecf114164"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interactive Econ Lab" sheetId="10" r:id="Rd59d8974eca346bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Lab" sheetId="11" r:id="R7d4d4114a8224a4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R588e4e673e034f30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rd4c38f78daa2495d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Data" sheetId="3" r:id="R524dc63d6911419e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression" sheetId="4" r:id="R2eeb380ef8b14452"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Notes" sheetId="5" r:id="R721219ec4b6242bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart Data" sheetId="6" r:id="R142620cc38a8456d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Dashboard" sheetId="7" r:id="R9e8581c6f467450e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Data" sheetId="8" r:id="Re71c0963dc494025"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Models" sheetId="9" r:id="R427acdc95bf44fba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interactive Econ Lab" sheetId="10" r:id="R2ac410179e67405b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Lab" sheetId="11" r:id="R5d1325d2075247b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Scorecard" sheetId="12" r:id="R789897d739764a7f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -38,7 +39,7 @@
     <x:numFmt numFmtId="211" formatCode="+0%;-0%;0%"/>
     <x:numFmt numFmtId="212" formatCode="+0.0%;-0.0%;0.0%"/>
   </x:numFmts>
-  <x:fonts count="21">
+  <x:fonts count="23">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -154,6 +155,18 @@
     <x:font>
       <x:b/>
       <x:sz val="16"/>
+      <x:color rgb="FF17324D"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="22"/>
+      <x:color rgb="FF17324D"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
       <x:color rgb="FF17324D"/>
       <x:name val="Carlito"/>
     </x:font>
@@ -465,7 +478,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="365">
+  <x:cellXfs count="457">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1207,6 +1220,224 @@
       <x:alignment horizontal="center"/>
     </x:xf>
     <x:xf numFmtId="212" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="21" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="21" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="21" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="21" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="21" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="21" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="21" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="21" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1854,6 +2085,121 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/drawings/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:t>Selected state's loss per person, 2022–2025</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:plotArea>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Loss per person</c:v>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'State Scorecard'!$A$18:$A$21</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'State Scorecard'!$D$18:$D$21</c:f>
+              <c:numCache>
+                <c:formatCode>$0</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:smooth val="0"/>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="48672768"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="$0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
@@ -1880,7 +2226,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3b04e7e3992449ce"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R77fd5d04071f4848"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1910,7 +2256,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4f97da1c400a4646"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R27eeb534ee424324"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1945,7 +2291,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6062a277b44c445f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9904067822b342bc"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1980,7 +2326,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re34d5bea8cef4c8a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfa1a549b485b41b1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2015,7 +2361,42 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R31146cf556f54f5e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra9b412032f324d80"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7cecbc794568407c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2411,10 +2792,10 @@
       <x:c r="H7" s="30"/>
       <x:c r="I7" s="31"/>
       <x:c r="K7" s="57" t="str">
-        <x:v>1. Open Interactive Econ Lab
-2. Compare states and outcomes
-3. Open Scenario Lab
-4. Test an income-change scenario
+        <x:v>1. Compare states in Interactive Econ Lab
+2. Build a profile in State Scorecard
+3. Test an income scenario
+4. Read the evidence verdict
 5. Check Sources &amp; Notes</x:v>
       </x:c>
       <x:c r="L7" s="58"/>
@@ -3263,7 +3644,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf59289ecaef47d3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15e62950b72a4b61"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -3747,7 +4128,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf55c8bf5eebd4686"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19c58797e2e74e66"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -3760,6 +4141,503 @@
             </x14:dataBar>
           </x14:cfRule>
           <xm:sqref>E12:E14</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </x:ext>
+  </x:extLst>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="324" t="str">
+        <x:v>STATE SCORECARD — EXPOSURE, SEVERITY, AND ECONOMIC HARM</x:v>
+      </x:c>
+      <x:c r="B1" s="324"/>
+      <x:c r="C1" s="324"/>
+      <x:c r="D1" s="324"/>
+      <x:c r="E1" s="324"/>
+      <x:c r="F1" s="324"/>
+      <x:c r="G1" s="324"/>
+      <x:c r="H1" s="324"/>
+      <x:c r="I1" s="324"/>
+      <x:c r="J1" s="324"/>
+      <x:c r="K1" s="324"/>
+      <x:c r="L1" s="324"/>
+      <x:c r="M1" s="324"/>
+      <x:c r="N1" s="324"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="324"/>
+      <x:c r="B2" s="324"/>
+      <x:c r="C2" s="324"/>
+      <x:c r="D2" s="324"/>
+      <x:c r="E2" s="324"/>
+      <x:c r="F2" s="324"/>
+      <x:c r="G2" s="324"/>
+      <x:c r="H2" s="324"/>
+      <x:c r="I2" s="324"/>
+      <x:c r="J2" s="324"/>
+      <x:c r="K2" s="324"/>
+      <x:c r="L2" s="324"/>
+      <x:c r="M2" s="324"/>
+      <x:c r="N2" s="324"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="6" t="str">
+        <x:v>Choose a state and year. Percentiles compare the selected jurisdiction with all 50 states and Washington, D.C. in that year.</x:v>
+      </x:c>
+      <x:c r="B3" s="6"/>
+      <x:c r="C3" s="6"/>
+      <x:c r="D3" s="6"/>
+      <x:c r="E3" s="6"/>
+      <x:c r="F3" s="6"/>
+      <x:c r="G3" s="6"/>
+      <x:c r="H3" s="6"/>
+      <x:c r="I3" s="6"/>
+      <x:c r="J3" s="6"/>
+      <x:c r="K3" s="6"/>
+      <x:c r="L3" s="6"/>
+      <x:c r="M3" s="6"/>
+      <x:c r="N3" s="6"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="68" t="str">
+        <x:v>State</x:v>
+      </x:c>
+      <x:c r="B5" s="68"/>
+      <x:c r="C5" s="68"/>
+      <x:c r="D5" s="68" t="str">
+        <x:v>Year</x:v>
+      </x:c>
+      <x:c r="E5" s="68"/>
+      <x:c r="F5" s="68"/>
+      <x:c r="H5" s="37" t="str">
+        <x:v>LOSS / PERSON</x:v>
+      </x:c>
+      <x:c r="I5" s="37"/>
+      <x:c r="J5" s="37"/>
+      <x:c r="K5" s="37" t="str">
+        <x:v>MEDIAN INCOME</x:v>
+      </x:c>
+      <x:c r="L5" s="37"/>
+      <x:c r="M5" s="37"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="339" t="str">
+        <x:v>North Carolina</x:v>
+      </x:c>
+      <x:c r="B6" s="340"/>
+      <x:c r="C6" s="341"/>
+      <x:c r="D6" s="339" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="E6" s="340"/>
+      <x:c r="F6" s="341"/>
+      <x:c r="H6" s="380" t="n">
+        <x:f>SUMIFS('Panel Data'!$L$2:$L$205,'Panel Data'!$A$2:$A$205,$D$6,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
+        <x:v>39.06941683269926</x:v>
+      </x:c>
+      <x:c r="I6" s="381"/>
+      <x:c r="J6" s="382"/>
+      <x:c r="K6" s="389" t="n">
+        <x:f>SUMIFS('Panel Data'!$F$2:$F$205,'Panel Data'!$A$2:$A$205,$D$6,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
+        <x:v>73958</x:v>
+      </x:c>
+      <x:c r="L6" s="381"/>
+      <x:c r="M6" s="382"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="342"/>
+      <x:c r="B7" s="343"/>
+      <x:c r="C7" s="344"/>
+      <x:c r="D7" s="342"/>
+      <x:c r="E7" s="343"/>
+      <x:c r="F7" s="344"/>
+      <x:c r="H7" s="383"/>
+      <x:c r="I7" s="384"/>
+      <x:c r="J7" s="385"/>
+      <x:c r="K7" s="383"/>
+      <x:c r="L7" s="384"/>
+      <x:c r="M7" s="385"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="H9" s="365" t="str">
+        <x:v>PROFILE QUADRANT</x:v>
+      </x:c>
+      <x:c r="I9" s="365"/>
+      <x:c r="J9" s="365"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="390" t="str">
+        <x:v>Economic dimension</x:v>
+      </x:c>
+      <x:c r="B10" s="390" t="str">
+        <x:v>Selected value</x:v>
+      </x:c>
+      <x:c r="C10" s="390" t="str">
+        <x:v>Percentile</x:v>
+      </x:c>
+      <x:c r="D10" s="390" t="str">
+        <x:v>Interpretation</x:v>
+      </x:c>
+      <x:c r="E10" s="390" t="str">
+        <x:v>Rank / 51</x:v>
+      </x:c>
+      <x:c r="H10" s="418" t="str">
+        <x:f>IF(C11&gt;=0.5,IF(C12&gt;=0.5,"HIGH EXPOSURE / HIGH SEVERITY","HIGH EXPOSURE / LOWER SEVERITY"),IF(C12&gt;=0.5,"LOWER EXPOSURE / HIGH SEVERITY","LOWER EXPOSURE / LOWER SEVERITY"))</x:f>
+        <x:v>LOWER EXPOSURE / LOWER SEVERITY</x:v>
+      </x:c>
+      <x:c r="I10" s="419"/>
+      <x:c r="J10" s="419"/>
+      <x:c r="K10" s="419"/>
+      <x:c r="L10" s="419"/>
+      <x:c r="M10" s="420"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>Reported exposure</x:v>
+      </x:c>
+      <x:c r="B11" s="318" t="n">
+        <x:f>SUMIFS('Panel Data'!$K$2:$K$205,'Panel Data'!$A$2:$A$205,$D$6,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
+        <x:v>234.835629544169</x:v>
+      </x:c>
+      <x:c r="C11" s="69" t="n">
+        <x:f>1-COUNTIFS('Panel Data'!$A$2:$A$205,$D$6,'Panel Data'!$K$2:$K$205,"&gt;"&amp;B11)/50</x:f>
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:f>IF(C11&gt;=0.75,"High",IF(C11&gt;=0.25,"Middle","Low"))</x:f>
+        <x:v>Middle</x:v>
+      </x:c>
+      <x:c r="E11" t="n">
+        <x:f>1+COUNTIFS('Panel Data'!$A$2:$A$205,$D$6,'Panel Data'!$K$2:$K$205,"&gt;"&amp;B11)</x:f>
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="H11" s="421"/>
+      <x:c r="I11" s="422"/>
+      <x:c r="J11" s="422"/>
+      <x:c r="K11" s="422"/>
+      <x:c r="L11" s="422"/>
+      <x:c r="M11" s="423"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>Loss severity</x:v>
+      </x:c>
+      <x:c r="B12" s="226" t="n">
+        <x:f>SUMIFS('Panel Data'!$M$2:$M$205,'Panel Data'!$A$2:$A$205,$D$6,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
+        <x:v>16636.92043176561</x:v>
+      </x:c>
+      <x:c r="C12" s="69" t="n">
+        <x:f>1-COUNTIFS('Panel Data'!$A$2:$A$205,$D$6,'Panel Data'!$M$2:$M$205,"&gt;"&amp;B12)/50</x:f>
+        <x:v>0.28</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:f>IF(C12&gt;=0.75,"High",IF(C12&gt;=0.25,"Middle","Low"))</x:f>
+        <x:v>Middle</x:v>
+      </x:c>
+      <x:c r="E12" t="n">
+        <x:f>1+COUNTIFS('Panel Data'!$A$2:$A$205,$D$6,'Panel Data'!$M$2:$M$205,"&gt;"&amp;B12)</x:f>
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="H12" s="424"/>
+      <x:c r="I12" s="425"/>
+      <x:c r="J12" s="425"/>
+      <x:c r="K12" s="425"/>
+      <x:c r="L12" s="425"/>
+      <x:c r="M12" s="426"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>Overall harm</x:v>
+      </x:c>
+      <x:c r="B13" s="225" t="n">
+        <x:f>$H$6</x:f>
+        <x:v>39.06941683269926</x:v>
+      </x:c>
+      <x:c r="C13" s="69" t="n">
+        <x:f>1-COUNTIFS('Panel Data'!$A$2:$A$205,$D$6,'Panel Data'!$L$2:$L$205,"&gt;"&amp;B13)/50</x:f>
+        <x:v>0.28</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:f>IF(C13&gt;=0.75,"High",IF(C13&gt;=0.25,"Middle","Low"))</x:f>
+        <x:v>Middle</x:v>
+      </x:c>
+      <x:c r="E13" t="n">
+        <x:f>1+COUNTIFS('Panel Data'!$A$2:$A$205,$D$6,'Panel Data'!$L$2:$L$205,"&gt;"&amp;B13)</x:f>
+        <x:v>37</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="67" t="str">
+        <x:v>FOUR-YEAR PROFILE</x:v>
+      </x:c>
+      <x:c r="B16" s="67"/>
+      <x:c r="C16" s="67"/>
+      <x:c r="D16" s="67"/>
+      <x:c r="E16" s="67"/>
+      <x:c r="F16" s="67"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="224" t="str">
+        <x:v>Year</x:v>
+      </x:c>
+      <x:c r="B17" s="224" t="str">
+        <x:v>Exposure</x:v>
+      </x:c>
+      <x:c r="C17" s="224" t="str">
+        <x:v>Severity</x:v>
+      </x:c>
+      <x:c r="D17" s="224" t="str">
+        <x:v>Loss / person</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="B18" s="318" t="n">
+        <x:f>SUMIFS('Panel Data'!$K$2:$K$205,'Panel Data'!$A$2:$A$205,$A18,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
+        <x:v>100.02689751138311</x:v>
+      </x:c>
+      <x:c r="C18" s="226" t="n">
+        <x:f>SUMIFS('Panel Data'!$M$2:$M$205,'Panel Data'!$A$2:$A$205,$A18,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
+        <x:v>16624.45859389805</x:v>
+      </x:c>
+      <x:c r="D18" s="225" t="n">
+        <x:f>SUMIFS('Panel Data'!$L$2:$L$205,'Panel Data'!$A$2:$A$205,$A18,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
+        <x:v>16.628930159540722</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="B19" s="318" t="n">
+        <x:f>SUMIFS('Panel Data'!$K$2:$K$205,'Panel Data'!$A$2:$A$205,$A19,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
+        <x:v>114.79606500549166</x:v>
+      </x:c>
+      <x:c r="C19" s="226" t="n">
+        <x:f>SUMIFS('Panel Data'!$M$2:$M$205,'Panel Data'!$A$2:$A$205,$A19,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
+        <x:v>19131.43120013027</x:v>
+      </x:c>
+      <x:c r="D19" s="225" t="n">
+        <x:f>SUMIFS('Panel Data'!$L$2:$L$205,'Panel Data'!$A$2:$A$205,$A19,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
+        <x:v>21.962130196982457</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="B20" s="318" t="n">
+        <x:f>SUMIFS('Panel Data'!$K$2:$K$205,'Panel Data'!$A$2:$A$205,$A20,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
+        <x:v>203.2302920098406</x:v>
+      </x:c>
+      <x:c r="C20" s="226" t="n">
+        <x:f>SUMIFS('Panel Data'!$M$2:$M$205,'Panel Data'!$A$2:$A$205,$A20,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
+        <x:v>14726.304300440488</x:v>
+      </x:c>
+      <x:c r="D20" s="225" t="n">
+        <x:f>SUMIFS('Panel Data'!$L$2:$L$205,'Panel Data'!$A$2:$A$205,$A20,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
+        <x:v>29.928311232042923</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="B21" s="318" t="n">
+        <x:f>SUMIFS('Panel Data'!$K$2:$K$205,'Panel Data'!$A$2:$A$205,$A21,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
+        <x:v>234.835629544169</x:v>
+      </x:c>
+      <x:c r="C21" s="226" t="n">
+        <x:f>SUMIFS('Panel Data'!$M$2:$M$205,'Panel Data'!$A$2:$A$205,$A21,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
+        <x:v>16636.92043176561</x:v>
+      </x:c>
+      <x:c r="D21" s="225" t="n">
+        <x:f>SUMIFS('Panel Data'!$L$2:$L$205,'Panel Data'!$A$2:$A$205,$A21,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
+        <x:v>39.06941683269926</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="445" t="str">
+        <x:v>ECONOMIC READING
+Exposure measures how often residents report fraud; severity measures the average dollars lost per complaint. The quadrant prevents a single ranking from hiding the mechanism. A state can experience high total harm because exposure is elevated, losses are severe, or both.</x:v>
+      </x:c>
+      <x:c r="B24" s="446"/>
+      <x:c r="C24" s="446"/>
+      <x:c r="D24" s="446"/>
+      <x:c r="E24" s="447"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="448"/>
+      <x:c r="B25" s="449"/>
+      <x:c r="C25" s="449"/>
+      <x:c r="D25" s="449"/>
+      <x:c r="E25" s="450"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="448"/>
+      <x:c r="B26" s="449"/>
+      <x:c r="C26" s="449"/>
+      <x:c r="D26" s="449"/>
+      <x:c r="E26" s="450"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="448"/>
+      <x:c r="B27" s="449"/>
+      <x:c r="C27" s="449"/>
+      <x:c r="D27" s="449"/>
+      <x:c r="E27" s="450"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="451"/>
+      <x:c r="B28" s="452"/>
+      <x:c r="C28" s="452"/>
+      <x:c r="D28" s="452"/>
+      <x:c r="E28" s="453"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="456" t="str">
+        <x:v>CHALLENGE: Find one state with high exposure but lower severity, then another with lower exposure but high severity. What different prevention strategies might each profile suggest?</x:v>
+      </x:c>
+      <x:c r="B31" s="456"/>
+      <x:c r="C31" s="456"/>
+      <x:c r="D31" s="456"/>
+      <x:c r="E31" s="456"/>
+      <x:c r="F31" s="456"/>
+      <x:c r="G31" s="456"/>
+      <x:c r="H31" s="456"/>
+      <x:c r="I31" s="456"/>
+      <x:c r="J31" s="456"/>
+      <x:c r="K31" s="456"/>
+      <x:c r="L31" s="456"/>
+      <x:c r="M31" s="456"/>
+      <x:c r="N31" s="456"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="456"/>
+      <x:c r="B32" s="456"/>
+      <x:c r="C32" s="456"/>
+      <x:c r="D32" s="456"/>
+      <x:c r="E32" s="456"/>
+      <x:c r="F32" s="456"/>
+      <x:c r="G32" s="456"/>
+      <x:c r="H32" s="456"/>
+      <x:c r="I32" s="456"/>
+      <x:c r="J32" s="456"/>
+      <x:c r="K32" s="456"/>
+      <x:c r="L32" s="456"/>
+      <x:c r="M32" s="456"/>
+      <x:c r="N32" s="456"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="456"/>
+      <x:c r="B33" s="456"/>
+      <x:c r="C33" s="456"/>
+      <x:c r="D33" s="456"/>
+      <x:c r="E33" s="456"/>
+      <x:c r="F33" s="456"/>
+      <x:c r="G33" s="456"/>
+      <x:c r="H33" s="456"/>
+      <x:c r="I33" s="456"/>
+      <x:c r="J33" s="456"/>
+      <x:c r="K33" s="456"/>
+      <x:c r="L33" s="456"/>
+      <x:c r="M33" s="456"/>
+      <x:c r="N33" s="456"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="456"/>
+      <x:c r="B34" s="456"/>
+      <x:c r="C34" s="456"/>
+      <x:c r="D34" s="456"/>
+      <x:c r="E34" s="456"/>
+      <x:c r="F34" s="456"/>
+      <x:c r="G34" s="456"/>
+      <x:c r="H34" s="456"/>
+      <x:c r="I34" s="456"/>
+      <x:c r="J34" s="456"/>
+      <x:c r="K34" s="456"/>
+      <x:c r="L34" s="456"/>
+      <x:c r="M34" s="456"/>
+      <x:c r="N34" s="456"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:N2"/>
+    <x:mergeCell ref="A3:N3"/>
+    <x:mergeCell ref="A5:C5"/>
+    <x:mergeCell ref="D5:F5"/>
+    <x:mergeCell ref="A6:C7"/>
+    <x:mergeCell ref="D6:F7"/>
+    <x:mergeCell ref="H5:J5"/>
+    <x:mergeCell ref="K5:M5"/>
+    <x:mergeCell ref="H9:J9"/>
+    <x:mergeCell ref="H6:J7"/>
+    <x:mergeCell ref="K6:M7"/>
+    <x:mergeCell ref="H10:M12"/>
+    <x:mergeCell ref="A16:F16"/>
+    <x:mergeCell ref="A24:E28"/>
+    <x:mergeCell ref="A31:N34"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="C11:C13">
+    <x:cfRule type="dataBar" priority="1">
+      <x:dataBar>
+        <x:cfvo type="min"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FF2A9D8F"/>
+      </x:dataBar>
+      <x:extLst>
+        <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{145E6682-420D-8C48-59AD-7E3EAA9F4932}</x14:id>
+        </x:ext>
+      </x:extLst>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="A6">
+      <x:formula1>'Chart Data'!$A$2:$A$52</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D6">
+      <x:formula1>"2022,2023,2024,2025"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde693909820d40e7"/>
+  <x:extLst>
+    <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting>
+          <x14:cfRule type="dataBar" priority="1" id="{145E6682-420D-8C48-59AD-7E3EAA9F4932}">
+            <x14:dataBar gradient="1">
+              <x14:cfvo type="min"/>
+              <x14:cfvo type="max"/>
+              <x14:fillColor rgb="FF2A9D8F"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>C11:C13</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </x:ext>
@@ -4175,7 +5053,7 @@
     <x:mergeCell ref="A40:N42"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc07663cb080845fa"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R592b6cd1415f4858"/>
 </x:worksheet>
 </file>
 
@@ -7279,7 +8157,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba01d9a565d24c64"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffffefc08f594fd8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7696,7 +8574,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7baa045060714aa2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec3c4fdc53af47ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8974,7 +9852,7 @@
     <x:mergeCell ref="A30:N33"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra29926aca0334437"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ba04e64ad6a4412"/>
 </x:worksheet>
 </file>
 
@@ -19249,7 +20127,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d9aa9fb2b4a4a1e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8203d6b9d662439f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19814,7 +20692,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68efd47c9c144a3b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0cf2a0b489e45ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refine workbook visual system
Soften accent and input colors, standardize chart typography, and reduce visual weight across the interactive experience.
</commit_message>
<xml_diff>
--- a/Scam_Geography_Interactive_Economics_Project.xlsx
+++ b/Scam_Geography_Interactive_Economics_Project.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R891e676befcc4191"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interactive Econ Lab" sheetId="2" r:id="R2ed76975595b44a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Scorecard" sheetId="3" r:id="Rf666e9c8c0564ff2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Lab" sheetId="4" r:id="R3e91fba1764b458d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" r:id="R32c416821b5c4103"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Dashboard" sheetId="6" r:id="R7169e961d370424e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Data" sheetId="7" r:id="R93a9dd9bb83a4211"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Data" sheetId="8" r:id="R765154c8114240df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression" sheetId="9" r:id="R20406f7e4aaf47c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Models" sheetId="10" r:id="Rb9de9e362e0241c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Notes" sheetId="11" r:id="R23b8186c56df40a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart Data" sheetId="12" r:id="Rdce4a43154a042b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R07560b7f7cf440d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interactive Econ Lab" sheetId="2" r:id="R88072faed6df4a52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Scorecard" sheetId="3" r:id="R1a9346fb4d884a83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Lab" sheetId="4" r:id="R690780ffe10f4201"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" r:id="Rc45d08b2af50465c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Dashboard" sheetId="6" r:id="R4c8bcb816bec4f2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Data" sheetId="7" r:id="R94e59058d568455d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Data" sheetId="8" r:id="Rfa2a6923d3804b84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression" sheetId="9" r:id="Ra6354884177d4a95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Models" sheetId="10" r:id="R3cd760b4116b4d18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Notes" sheetId="11" r:id="R74e4500ef8cf4383"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart Data" sheetId="12" r:id="Rd7b87286befc4947"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -185,7 +185,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFDDF25A"/>
+        <x:fgColor rgb="FFE4EDCF"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -230,7 +230,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF3A6"/>
+        <x:fgColor rgb="FFFFF6D8"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -411,44 +411,44 @@
       </x:top>
     </x:border>
     <x:border>
-      <x:left style="medium">
+      <x:left style="thin">
         <x:color rgb="FFD99B2B"/>
       </x:left>
-      <x:top style="medium">
+      <x:top style="thin">
         <x:color rgb="FFD99B2B"/>
       </x:top>
     </x:border>
     <x:border>
-      <x:top style="medium">
+      <x:top style="thin">
         <x:color rgb="FFD99B2B"/>
       </x:top>
     </x:border>
     <x:border>
-      <x:right style="medium">
+      <x:right style="thin">
         <x:color rgb="FFD99B2B"/>
       </x:right>
-      <x:top style="medium">
+      <x:top style="thin">
         <x:color rgb="FFD99B2B"/>
       </x:top>
     </x:border>
     <x:border>
-      <x:left style="medium">
+      <x:left style="thin">
         <x:color rgb="FFD99B2B"/>
       </x:left>
-      <x:bottom style="medium">
+      <x:bottom style="thin">
         <x:color rgb="FFD99B2B"/>
       </x:bottom>
     </x:border>
     <x:border>
-      <x:bottom style="medium">
+      <x:bottom style="thin">
         <x:color rgb="FFD99B2B"/>
       </x:bottom>
     </x:border>
     <x:border>
-      <x:right style="medium">
+      <x:right style="thin">
         <x:color rgb="FFD99B2B"/>
       </x:right>
-      <x:bottom style="medium">
+      <x:bottom style="thin">
         <x:color rgb="FFD99B2B"/>
       </x:bottom>
     </x:border>
@@ -1481,12 +1481,22 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
+              <a:rPr sz="900"/>
               <a:t>Selected outcome across time</a:t>
             </a:r>
           </a:p>
         </c:rich>
       </c:tx>
       <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="900"/>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
     </c:title>
     <c:plotArea>
       <c:lineChart>
@@ -1628,12 +1638,22 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
+              <a:rPr sz="900"/>
               <a:t>Selected state's loss per person, 2022–2025</a:t>
             </a:r>
           </a:p>
         </c:rich>
       </c:tx>
       <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="900"/>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
     </c:title>
     <c:plotArea>
       <c:lineChart>
@@ -1743,12 +1763,22 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
+              <a:rPr sz="900"/>
               <a:t>How model choice changes the scenario</a:t>
             </a:r>
           </a:p>
         </c:rich>
       </c:tx>
       <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="900"/>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
     </c:title>
     <c:plotArea>
       <c:barChart>
@@ -1881,12 +1911,22 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
+              <a:rPr sz="900"/>
               <a:t>Highest reported loss per capita (2025)</a:t>
             </a:r>
           </a:p>
         </c:rich>
       </c:tx>
       <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="900"/>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
     </c:title>
     <c:plotArea>
       <c:barChart>
@@ -1991,12 +2031,22 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
+              <a:rPr sz="900"/>
               <a:t>Higher-income states tend to report larger losses per resident</a:t>
             </a:r>
           </a:p>
         </c:rich>
       </c:tx>
       <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="900"/>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
     </c:title>
     <c:plotArea>
       <c:scatterChart>
@@ -2097,12 +2147,22 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
+              <a:rPr sz="900"/>
               <a:t>Reported loss per resident nearly doubled, 2022–2025</a:t>
             </a:r>
           </a:p>
         </c:rich>
       </c:tx>
       <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="900"/>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
     </c:title>
     <c:plotArea>
       <c:lineChart>
@@ -2226,7 +2286,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R860d2a14e588415d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1b919ba3124b42fc"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2261,7 +2321,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb003b5a0ae664589"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbac33135aebd483d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2296,7 +2356,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0ca7bb60673f4ff1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc3209e7d2246495d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2331,7 +2391,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rddf3d3fa670c4576"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8cab3612050a414f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2361,7 +2421,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3b0e5e0aaa0346e7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3f400ae8979f4703"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2396,7 +2456,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0ffaa9b25a264c1b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re1433aab35ea4881"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3706,7 +3766,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfed9fe3b62c04dc6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda336d38c0024b14"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4982,7 +5042,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2540b6b1aa7c4cc7"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f7c2d75774c4a15"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -5479,7 +5539,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R835d599547ba4d16"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce81485bf7164b44"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -5963,7 +6023,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R794dd8c6e5d343e3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a2c722445934657"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -6391,7 +6451,7 @@
     <x:mergeCell ref="A40:N42"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1964bf63daf4b20"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R685c14d942a84026"/>
 </x:worksheet>
 </file>
 
@@ -6901,7 +6961,7 @@
     <x:mergeCell ref="A30:N33"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf34c4746babd4c9d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1b5b7e860cb4a52"/>
 </x:worksheet>
 </file>
 
@@ -10005,7 +10065,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18a8db29cf2941cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8da9eb0600c412b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20281,7 +20341,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R357f523ee6cf4c4e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64c5bc17a1cb4665"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20698,7 +20758,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1db6f2e7ccad48f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7c59e62c9324a73"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete portfolio-grade workbook polish
Add responsive scorecard states, clarify interactive guidance, fix clipped prompt content, and restore the complete regional panel display.
</commit_message>
<xml_diff>
--- a/Scam_Geography_Interactive_Economics_Project.xlsx
+++ b/Scam_Geography_Interactive_Economics_Project.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R07560b7f7cf440d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interactive Econ Lab" sheetId="2" r:id="R88072faed6df4a52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Scorecard" sheetId="3" r:id="R1a9346fb4d884a83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Lab" sheetId="4" r:id="R690780ffe10f4201"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" r:id="Rc45d08b2af50465c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Dashboard" sheetId="6" r:id="R4c8bcb816bec4f2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Data" sheetId="7" r:id="R94e59058d568455d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Data" sheetId="8" r:id="Rfa2a6923d3804b84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression" sheetId="9" r:id="Ra6354884177d4a95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Models" sheetId="10" r:id="R3cd760b4116b4d18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Notes" sheetId="11" r:id="R74e4500ef8cf4383"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart Data" sheetId="12" r:id="Rd7b87286befc4947"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Re3267b9c02d2469a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interactive Econ Lab" sheetId="2" r:id="R81995f3df5a14089"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Scorecard" sheetId="3" r:id="Rd570963bebc843f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Lab" sheetId="4" r:id="R60ea0c275cab4988"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" r:id="R6dc29620f4814471"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Dashboard" sheetId="6" r:id="R1eb387e44e1d42e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Data" sheetId="7" r:id="R77f616f387e8481f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Data" sheetId="8" r:id="R54ed324b5d2047be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression" sheetId="9" r:id="Rb30f5e8f3d494ff5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Models" sheetId="10" r:id="R349598b681fe4031"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Notes" sheetId="11" r:id="R1d10a625128340a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart Data" sheetId="12" r:id="R1d253b4704784fbb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -234,7 +234,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="36">
+  <x:borders count="44">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -454,6 +454,58 @@
     </x:border>
     <x:border>
       <x:left style="thin">
+        <x:color rgb="FF17324D"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FF17324D"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FF17324D"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FF17324D"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF17324D"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF17324D"/>
+      </x:left>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FF17324D"/>
+      </x:right>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF17324D"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FF17324D"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FF17324D"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FF17324D"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FF17324D"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
         <x:color rgb="FFC5D3DC"/>
       </x:left>
       <x:top style="thin">
@@ -478,7 +530,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="457">
+  <x:cellXfs count="525">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1126,12 +1178,60 @@
     </x:xf>
     <x:xf numFmtId="207" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="204" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="205" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="205" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="205" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="205" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1185,17 +1285,129 @@
     <x:xf numFmtId="210" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="211" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="2" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1211,12 +1423,12 @@
     <x:xf numFmtId="205" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="203" fontId="20" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="205" fontId="20" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="203" fontId="20" fillId="6" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="205" fontId="20" fillId="6" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="203" fontId="20" fillId="6" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="203" fontId="20" fillId="6" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="20" fillId="6" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="20" fillId="6" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
-    <x:xf numFmtId="205" fontId="20" fillId="6" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="205" fontId="20" fillId="6" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
     <x:xf numFmtId="212" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1442,7 +1654,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="2">
+  <x:dxfs count="9">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -1462,6 +1674,82 @@
       <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFDFF2E8"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF17324D"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFBE7C6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF17324D"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFEAF1F5"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF17324D"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE4EDCF"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF17324D"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFBE7C6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF17324D"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF1C9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF17324D"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFDCECF4"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF17324D"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE4EDCF"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -2286,7 +2574,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1b919ba3124b42fc"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R432b1023d8e74f7a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2321,7 +2609,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbac33135aebd483d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R929337fa44844875"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2356,7 +2644,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc3209e7d2246495d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3c6d0db1a44647dd"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2391,7 +2679,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8cab3612050a414f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6e25043340ae4e1b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2421,7 +2709,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3f400ae8979f4703"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R342b0701f4ce46b1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2456,7 +2744,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re1433aab35ea4881"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R857b8bcf8a8543f2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3766,7 +4054,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda336d38c0024b14"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R102b0bbd7e8a4a56"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4559,42 +4847,42 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="324" t="str">
+      <x:c r="A1" s="344" t="str">
         <x:v>SCAM GEOGRAPHY — INTERACTIVE ECONOMICS LAB</x:v>
       </x:c>
-      <x:c r="B1" s="324"/>
-      <x:c r="C1" s="324"/>
-      <x:c r="D1" s="324"/>
-      <x:c r="E1" s="324"/>
-      <x:c r="F1" s="324"/>
-      <x:c r="G1" s="324"/>
-      <x:c r="H1" s="324"/>
-      <x:c r="I1" s="324"/>
-      <x:c r="J1" s="324"/>
-      <x:c r="K1" s="324"/>
-      <x:c r="L1" s="324"/>
-      <x:c r="M1" s="324"/>
-      <x:c r="N1" s="324"/>
+      <x:c r="B1" s="344"/>
+      <x:c r="C1" s="344"/>
+      <x:c r="D1" s="344"/>
+      <x:c r="E1" s="344"/>
+      <x:c r="F1" s="344"/>
+      <x:c r="G1" s="344"/>
+      <x:c r="H1" s="344"/>
+      <x:c r="I1" s="344"/>
+      <x:c r="J1" s="344"/>
+      <x:c r="K1" s="344"/>
+      <x:c r="L1" s="344"/>
+      <x:c r="M1" s="344"/>
+      <x:c r="N1" s="344"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="324"/>
-      <x:c r="B2" s="324"/>
-      <x:c r="C2" s="324"/>
-      <x:c r="D2" s="324"/>
-      <x:c r="E2" s="324"/>
-      <x:c r="F2" s="324"/>
-      <x:c r="G2" s="324"/>
-      <x:c r="H2" s="324"/>
-      <x:c r="I2" s="324"/>
-      <x:c r="J2" s="324"/>
-      <x:c r="K2" s="324"/>
-      <x:c r="L2" s="324"/>
-      <x:c r="M2" s="324"/>
-      <x:c r="N2" s="324"/>
+      <x:c r="A2" s="344"/>
+      <x:c r="B2" s="344"/>
+      <x:c r="C2" s="344"/>
+      <x:c r="D2" s="344"/>
+      <x:c r="E2" s="344"/>
+      <x:c r="F2" s="344"/>
+      <x:c r="G2" s="344"/>
+      <x:c r="H2" s="344"/>
+      <x:c r="I2" s="344"/>
+      <x:c r="J2" s="344"/>
+      <x:c r="K2" s="344"/>
+      <x:c r="L2" s="344"/>
+      <x:c r="M2" s="344"/>
+      <x:c r="N2" s="344"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="6" t="str">
-        <x:v>Change the yellow cells. Every result below updates from the 2022–2025 state panel.</x:v>
+        <x:v>Adjust the warm input cells. Every result below updates from the 2022–2025 state panel.</x:v>
       </x:c>
       <x:c r="B3" s="6"/>
       <x:c r="C3" s="6"/>
@@ -4633,40 +4921,40 @@
       <x:c r="L5" s="68"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="339" t="n">
+      <x:c r="A6" s="359" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="B6" s="340"/>
-      <x:c r="C6" s="341"/>
-      <x:c r="D6" s="339" t="str">
+      <x:c r="B6" s="360"/>
+      <x:c r="C6" s="361"/>
+      <x:c r="D6" s="359" t="str">
         <x:v>North Carolina</x:v>
       </x:c>
-      <x:c r="E6" s="340"/>
-      <x:c r="F6" s="341"/>
-      <x:c r="G6" s="339" t="str">
+      <x:c r="E6" s="360"/>
+      <x:c r="F6" s="361"/>
+      <x:c r="G6" s="359" t="str">
         <x:v>California</x:v>
       </x:c>
-      <x:c r="H6" s="340"/>
-      <x:c r="I6" s="341"/>
-      <x:c r="J6" s="339" t="str">
+      <x:c r="H6" s="360"/>
+      <x:c r="I6" s="361"/>
+      <x:c r="J6" s="359" t="str">
         <x:v>Loss per capita</x:v>
       </x:c>
-      <x:c r="K6" s="340"/>
-      <x:c r="L6" s="341"/>
+      <x:c r="K6" s="360"/>
+      <x:c r="L6" s="361"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="342"/>
-      <x:c r="B7" s="343"/>
-      <x:c r="C7" s="344"/>
-      <x:c r="D7" s="342"/>
-      <x:c r="E7" s="343"/>
-      <x:c r="F7" s="344"/>
-      <x:c r="G7" s="342"/>
-      <x:c r="H7" s="343"/>
-      <x:c r="I7" s="344"/>
-      <x:c r="J7" s="342"/>
-      <x:c r="K7" s="343"/>
-      <x:c r="L7" s="344"/>
+      <x:c r="A7" s="362"/>
+      <x:c r="B7" s="363"/>
+      <x:c r="C7" s="364"/>
+      <x:c r="D7" s="362"/>
+      <x:c r="E7" s="363"/>
+      <x:c r="F7" s="364"/>
+      <x:c r="G7" s="362"/>
+      <x:c r="H7" s="363"/>
+      <x:c r="I7" s="364"/>
+      <x:c r="J7" s="362"/>
+      <x:c r="K7" s="363"/>
+      <x:c r="L7" s="364"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="36" t="str">
@@ -4714,15 +5002,15 @@
         <x:f>$J$6</x:f>
         <x:v>Loss per capita</x:v>
       </x:c>
-      <x:c r="B11" s="345" t="n">
+      <x:c r="B11" s="365" t="n">
         <x:f>IF($J$6="Loss per capita",SUMIFS('Panel Data'!$L$2:$L$205,'Panel Data'!$A$2:$A$205,$A$6,'Panel Data'!$B$2:$B$205,$D$6),IF($J$6="Complaints per 100k",SUMIFS('Panel Data'!$K$2:$K$205,'Panel Data'!$A$2:$A$205,$A$6,'Panel Data'!$B$2:$B$205,$D$6),SUMIFS('Panel Data'!$M$2:$M$205,'Panel Data'!$A$2:$A$205,$A$6,'Panel Data'!$B$2:$B$205,$D$6)))</x:f>
         <x:v>39.06941683269926</x:v>
       </x:c>
-      <x:c r="C11" s="345" t="n">
+      <x:c r="C11" s="365" t="n">
         <x:f>IF($J$6="Loss per capita",SUMIFS('Panel Data'!$L$2:$L$205,'Panel Data'!$A$2:$A$205,$A$6,'Panel Data'!$B$2:$B$205,$G$6),IF($J$6="Complaints per 100k",SUMIFS('Panel Data'!$K$2:$K$205,'Panel Data'!$A$2:$A$205,$A$6,'Panel Data'!$B$2:$B$205,$G$6),SUMIFS('Panel Data'!$M$2:$M$205,'Panel Data'!$A$2:$A$205,$A$6,'Panel Data'!$B$2:$B$205,$G$6)))</x:f>
         <x:v>93.1929648056163</x:v>
       </x:c>
-      <x:c r="D11" s="346" t="n">
+      <x:c r="D11" s="366" t="n">
         <x:f>IFERROR(C11/B11-1,0)</x:f>
         <x:v>1.3853175286613997</x:v>
       </x:c>
@@ -4745,7 +5033,7 @@
         <x:f>SUMIFS('Panel Data'!$F$2:$F$205,'Panel Data'!$A$2:$A$205,$A$6,'Panel Data'!$B$2:$B$205,$G$6)</x:f>
         <x:v>100149</x:v>
       </x:c>
-      <x:c r="D12" s="346" t="n">
+      <x:c r="D12" s="366" t="n">
         <x:f>IFERROR(C12/B12-1,0)</x:f>
         <x:v>0.35413342708023476</x:v>
       </x:c>
@@ -4768,7 +5056,7 @@
         <x:f>SUMIFS('Panel Data'!$K$2:$K$205,'Panel Data'!$A$2:$A$205,$A$6,'Panel Data'!$B$2:$B$205,$G$6)</x:f>
         <x:v>295.23274463716774</x:v>
       </x:c>
-      <x:c r="D13" s="346" t="n">
+      <x:c r="D13" s="366" t="n">
         <x:f>IFERROR(C13/B13-1,0)</x:f>
         <x:v>0.25718889084349517</x:v>
       </x:c>
@@ -4791,7 +5079,7 @@
         <x:f>SUMIFS('Panel Data'!$M$2:$M$205,'Panel Data'!$A$2:$A$205,$A$6,'Panel Data'!$B$2:$B$205,$G$6)</x:f>
         <x:v>31565.931116532374</x:v>
       </x:c>
-      <x:c r="D14" s="346" t="n">
+      <x:c r="D14" s="366" t="n">
         <x:f>IFERROR(C14/B14-1,0)</x:f>
         <x:v>0.897342194187702</x:v>
       </x:c>
@@ -4829,11 +5117,11 @@
       <x:c r="A19" t="n">
         <x:v>2022</x:v>
       </x:c>
-      <x:c r="B19" s="345" t="n">
+      <x:c r="B19" s="365" t="n">
         <x:f>IF($J$6="Loss per capita",SUMIFS('Panel Data'!$L$2:$L$205,'Panel Data'!$A$2:$A$205,$A19,'Panel Data'!$B$2:$B$205,$D$6),IF($J$6="Complaints per 100k",SUMIFS('Panel Data'!$K$2:$K$205,'Panel Data'!$A$2:$A$205,$A19,'Panel Data'!$B$2:$B$205,$D$6),SUMIFS('Panel Data'!$M$2:$M$205,'Panel Data'!$A$2:$A$205,$A19,'Panel Data'!$B$2:$B$205,$D$6)))</x:f>
         <x:v>16.628930159540722</x:v>
       </x:c>
-      <x:c r="C19" s="345" t="n">
+      <x:c r="C19" s="365" t="n">
         <x:f>IF($J$6="Loss per capita",SUMIFS('Panel Data'!$L$2:$L$205,'Panel Data'!$A$2:$A$205,$A19,'Panel Data'!$B$2:$B$205,$G$6),IF($J$6="Complaints per 100k",SUMIFS('Panel Data'!$K$2:$K$205,'Panel Data'!$A$2:$A$205,$A19,'Panel Data'!$B$2:$B$205,$G$6),SUMIFS('Panel Data'!$M$2:$M$205,'Panel Data'!$A$2:$A$205,$A19,'Panel Data'!$B$2:$B$205,$G$6)))</x:f>
         <x:v>51.29760127444337</x:v>
       </x:c>
@@ -4842,11 +5130,11 @@
       <x:c r="A20" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="B20" s="345" t="n">
+      <x:c r="B20" s="365" t="n">
         <x:f>IF($J$6="Loss per capita",SUMIFS('Panel Data'!$L$2:$L$205,'Panel Data'!$A$2:$A$205,$A20,'Panel Data'!$B$2:$B$205,$D$6),IF($J$6="Complaints per 100k",SUMIFS('Panel Data'!$K$2:$K$205,'Panel Data'!$A$2:$A$205,$A20,'Panel Data'!$B$2:$B$205,$D$6),SUMIFS('Panel Data'!$M$2:$M$205,'Panel Data'!$A$2:$A$205,$A20,'Panel Data'!$B$2:$B$205,$D$6)))</x:f>
         <x:v>21.962130196982457</x:v>
       </x:c>
-      <x:c r="C20" s="345" t="n">
+      <x:c r="C20" s="365" t="n">
         <x:f>IF($J$6="Loss per capita",SUMIFS('Panel Data'!$L$2:$L$205,'Panel Data'!$A$2:$A$205,$A20,'Panel Data'!$B$2:$B$205,$G$6),IF($J$6="Complaints per 100k",SUMIFS('Panel Data'!$K$2:$K$205,'Panel Data'!$A$2:$A$205,$A20,'Panel Data'!$B$2:$B$205,$G$6),SUMIFS('Panel Data'!$M$2:$M$205,'Panel Data'!$A$2:$A$205,$A20,'Panel Data'!$B$2:$B$205,$G$6)))</x:f>
         <x:v>55.32900126781538</x:v>
       </x:c>
@@ -4855,11 +5143,11 @@
       <x:c r="A21" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="B21" s="345" t="n">
+      <x:c r="B21" s="365" t="n">
         <x:f>IF($J$6="Loss per capita",SUMIFS('Panel Data'!$L$2:$L$205,'Panel Data'!$A$2:$A$205,$A21,'Panel Data'!$B$2:$B$205,$D$6),IF($J$6="Complaints per 100k",SUMIFS('Panel Data'!$K$2:$K$205,'Panel Data'!$A$2:$A$205,$A21,'Panel Data'!$B$2:$B$205,$D$6),SUMIFS('Panel Data'!$M$2:$M$205,'Panel Data'!$A$2:$A$205,$A21,'Panel Data'!$B$2:$B$205,$D$6)))</x:f>
         <x:v>29.928311232042923</x:v>
       </x:c>
-      <x:c r="C21" s="345" t="n">
+      <x:c r="C21" s="365" t="n">
         <x:f>IF($J$6="Loss per capita",SUMIFS('Panel Data'!$L$2:$L$205,'Panel Data'!$A$2:$A$205,$A21,'Panel Data'!$B$2:$B$205,$G$6),IF($J$6="Complaints per 100k",SUMIFS('Panel Data'!$K$2:$K$205,'Panel Data'!$A$2:$A$205,$A21,'Panel Data'!$B$2:$B$205,$G$6),SUMIFS('Panel Data'!$M$2:$M$205,'Panel Data'!$A$2:$A$205,$A21,'Panel Data'!$B$2:$B$205,$G$6)))</x:f>
         <x:v>65.1617877268053</x:v>
       </x:c>
@@ -4868,11 +5156,11 @@
       <x:c r="A22" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="B22" s="345" t="n">
+      <x:c r="B22" s="365" t="n">
         <x:f>IF($J$6="Loss per capita",SUMIFS('Panel Data'!$L$2:$L$205,'Panel Data'!$A$2:$A$205,$A22,'Panel Data'!$B$2:$B$205,$D$6),IF($J$6="Complaints per 100k",SUMIFS('Panel Data'!$K$2:$K$205,'Panel Data'!$A$2:$A$205,$A22,'Panel Data'!$B$2:$B$205,$D$6),SUMIFS('Panel Data'!$M$2:$M$205,'Panel Data'!$A$2:$A$205,$A22,'Panel Data'!$B$2:$B$205,$D$6)))</x:f>
         <x:v>39.06941683269926</x:v>
       </x:c>
-      <x:c r="C22" s="345" t="n">
+      <x:c r="C22" s="365" t="n">
         <x:f>IF($J$6="Loss per capita",SUMIFS('Panel Data'!$L$2:$L$205,'Panel Data'!$A$2:$A$205,$A22,'Panel Data'!$B$2:$B$205,$G$6),IF($J$6="Complaints per 100k",SUMIFS('Panel Data'!$K$2:$K$205,'Panel Data'!$A$2:$A$205,$A22,'Panel Data'!$B$2:$B$205,$G$6),SUMIFS('Panel Data'!$M$2:$M$205,'Panel Data'!$A$2:$A$205,$A22,'Panel Data'!$B$2:$B$205,$G$6)))</x:f>
         <x:v>93.1929648056163</x:v>
       </x:c>
@@ -4929,69 +5217,97 @@
       </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="352" t="str">
-        <x:v>Try this:
+      <x:c r="A33" s="412" t="str">
+        <x:v>TRY THIS
 1. Compare North Carolina with California.
-2. Switch the outcome from loss/person to complaints/100K.
+2. Switch the outcome from loss per person to complaints per 100,000.
 3. Change the year.
 4. Explain whether exposure or severity drives the gap.</x:v>
       </x:c>
-      <x:c r="B33" s="352"/>
-      <x:c r="C33" s="352"/>
-      <x:c r="E33" s="349" t="str">
+      <x:c r="B33" s="413"/>
+      <x:c r="C33" s="414"/>
+      <x:c r="E33" s="385" t="str">
         <x:v>ECONOMICS VERDICT
 The between-state relationship is strong and survives outlier checks. The within-state estimate is imprecise, so this project supports a geographic association—not a causal claim that rising income produces fraud losses.</x:v>
       </x:c>
-      <x:c r="F33" s="349"/>
-      <x:c r="G33" s="349"/>
-      <x:c r="H33" s="349"/>
-      <x:c r="I33" s="349"/>
-      <x:c r="J33" s="349"/>
-      <x:c r="K33" s="349"/>
-      <x:c r="L33" s="349"/>
-      <x:c r="M33" s="349"/>
+      <x:c r="F33" s="386"/>
+      <x:c r="G33" s="386"/>
+      <x:c r="H33" s="386"/>
+      <x:c r="I33" s="386"/>
+      <x:c r="J33" s="386"/>
+      <x:c r="K33" s="386"/>
+      <x:c r="L33" s="386"/>
+      <x:c r="M33" s="387"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="352"/>
-      <x:c r="B34" s="352"/>
-      <x:c r="C34" s="352"/>
-      <x:c r="E34" s="349"/>
-      <x:c r="F34" s="349"/>
-      <x:c r="G34" s="349"/>
-      <x:c r="H34" s="349"/>
-      <x:c r="I34" s="349"/>
-      <x:c r="J34" s="349"/>
-      <x:c r="K34" s="349"/>
-      <x:c r="L34" s="349"/>
-      <x:c r="M34" s="349"/>
+      <x:c r="A34" s="415"/>
+      <x:c r="B34" s="416"/>
+      <x:c r="C34" s="417"/>
+      <x:c r="E34" s="388"/>
+      <x:c r="F34" s="389"/>
+      <x:c r="G34" s="389"/>
+      <x:c r="H34" s="389"/>
+      <x:c r="I34" s="389"/>
+      <x:c r="J34" s="389"/>
+      <x:c r="K34" s="389"/>
+      <x:c r="L34" s="389"/>
+      <x:c r="M34" s="390"/>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="352"/>
-      <x:c r="B35" s="352"/>
-      <x:c r="C35" s="352"/>
-      <x:c r="E35" s="349"/>
-      <x:c r="F35" s="349"/>
-      <x:c r="G35" s="349"/>
-      <x:c r="H35" s="349"/>
-      <x:c r="I35" s="349"/>
-      <x:c r="J35" s="349"/>
-      <x:c r="K35" s="349"/>
-      <x:c r="L35" s="349"/>
-      <x:c r="M35" s="349"/>
+      <x:c r="A35" s="415"/>
+      <x:c r="B35" s="416"/>
+      <x:c r="C35" s="417"/>
+      <x:c r="E35" s="388"/>
+      <x:c r="F35" s="389"/>
+      <x:c r="G35" s="389"/>
+      <x:c r="H35" s="389"/>
+      <x:c r="I35" s="389"/>
+      <x:c r="J35" s="389"/>
+      <x:c r="K35" s="389"/>
+      <x:c r="L35" s="389"/>
+      <x:c r="M35" s="390"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="352"/>
-      <x:c r="B36" s="352"/>
-      <x:c r="C36" s="352"/>
-      <x:c r="E36" s="349"/>
-      <x:c r="F36" s="349"/>
-      <x:c r="G36" s="349"/>
-      <x:c r="H36" s="349"/>
-      <x:c r="I36" s="349"/>
-      <x:c r="J36" s="349"/>
-      <x:c r="K36" s="349"/>
-      <x:c r="L36" s="349"/>
-      <x:c r="M36" s="349"/>
+      <x:c r="A36" s="415"/>
+      <x:c r="B36" s="416"/>
+      <x:c r="C36" s="417"/>
+      <x:c r="E36" s="388"/>
+      <x:c r="F36" s="389"/>
+      <x:c r="G36" s="389"/>
+      <x:c r="H36" s="389"/>
+      <x:c r="I36" s="389"/>
+      <x:c r="J36" s="389"/>
+      <x:c r="K36" s="389"/>
+      <x:c r="L36" s="389"/>
+      <x:c r="M36" s="390"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="415"/>
+      <x:c r="B37" s="416"/>
+      <x:c r="C37" s="417"/>
+      <x:c r="E37" s="388"/>
+      <x:c r="F37" s="389"/>
+      <x:c r="G37" s="389"/>
+      <x:c r="H37" s="389"/>
+      <x:c r="I37" s="389"/>
+      <x:c r="J37" s="389"/>
+      <x:c r="K37" s="389"/>
+      <x:c r="L37" s="389"/>
+      <x:c r="M37" s="390"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="418"/>
+      <x:c r="B38" s="419"/>
+      <x:c r="C38" s="420"/>
+      <x:c r="E38" s="391"/>
+      <x:c r="F38" s="392"/>
+      <x:c r="G38" s="392"/>
+      <x:c r="H38" s="392"/>
+      <x:c r="I38" s="392"/>
+      <x:c r="J38" s="392"/>
+      <x:c r="K38" s="392"/>
+      <x:c r="L38" s="392"/>
+      <x:c r="M38" s="393"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5010,8 +5326,8 @@
     <x:mergeCell ref="H10:M14"/>
     <x:mergeCell ref="A17:F17"/>
     <x:mergeCell ref="A25:C25"/>
-    <x:mergeCell ref="E33:M36"/>
-    <x:mergeCell ref="A33:C36"/>
+    <x:mergeCell ref="E33:M38"/>
+    <x:mergeCell ref="A33:C38"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="D11:D14">
     <x:cfRule type="dataBar" priority="1">
@@ -5042,7 +5358,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f7c2d75774c4a15"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18bf83056d0f4542"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -5083,38 +5399,38 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="324" t="str">
+      <x:c r="A1" s="344" t="str">
         <x:v>STATE SCORECARD — EXPOSURE, SEVERITY, AND ECONOMIC HARM</x:v>
       </x:c>
-      <x:c r="B1" s="324"/>
-      <x:c r="C1" s="324"/>
-      <x:c r="D1" s="324"/>
-      <x:c r="E1" s="324"/>
-      <x:c r="F1" s="324"/>
-      <x:c r="G1" s="324"/>
-      <x:c r="H1" s="324"/>
-      <x:c r="I1" s="324"/>
-      <x:c r="J1" s="324"/>
-      <x:c r="K1" s="324"/>
-      <x:c r="L1" s="324"/>
-      <x:c r="M1" s="324"/>
-      <x:c r="N1" s="324"/>
+      <x:c r="B1" s="344"/>
+      <x:c r="C1" s="344"/>
+      <x:c r="D1" s="344"/>
+      <x:c r="E1" s="344"/>
+      <x:c r="F1" s="344"/>
+      <x:c r="G1" s="344"/>
+      <x:c r="H1" s="344"/>
+      <x:c r="I1" s="344"/>
+      <x:c r="J1" s="344"/>
+      <x:c r="K1" s="344"/>
+      <x:c r="L1" s="344"/>
+      <x:c r="M1" s="344"/>
+      <x:c r="N1" s="344"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="324"/>
-      <x:c r="B2" s="324"/>
-      <x:c r="C2" s="324"/>
-      <x:c r="D2" s="324"/>
-      <x:c r="E2" s="324"/>
-      <x:c r="F2" s="324"/>
-      <x:c r="G2" s="324"/>
-      <x:c r="H2" s="324"/>
-      <x:c r="I2" s="324"/>
-      <x:c r="J2" s="324"/>
-      <x:c r="K2" s="324"/>
-      <x:c r="L2" s="324"/>
-      <x:c r="M2" s="324"/>
-      <x:c r="N2" s="324"/>
+      <x:c r="A2" s="344"/>
+      <x:c r="B2" s="344"/>
+      <x:c r="C2" s="344"/>
+      <x:c r="D2" s="344"/>
+      <x:c r="E2" s="344"/>
+      <x:c r="F2" s="344"/>
+      <x:c r="G2" s="344"/>
+      <x:c r="H2" s="344"/>
+      <x:c r="I2" s="344"/>
+      <x:c r="J2" s="344"/>
+      <x:c r="K2" s="344"/>
+      <x:c r="L2" s="344"/>
+      <x:c r="M2" s="344"/>
+      <x:c r="N2" s="344"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="6" t="str">
@@ -5157,75 +5473,75 @@
       <x:c r="M5" s="37"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="339" t="str">
+      <x:c r="A6" s="359" t="str">
         <x:v>North Carolina</x:v>
       </x:c>
-      <x:c r="B6" s="340"/>
-      <x:c r="C6" s="341"/>
-      <x:c r="D6" s="339" t="n">
+      <x:c r="B6" s="360"/>
+      <x:c r="C6" s="361"/>
+      <x:c r="D6" s="359" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="E6" s="340"/>
-      <x:c r="F6" s="341"/>
-      <x:c r="H6" s="380" t="n">
+      <x:c r="E6" s="360"/>
+      <x:c r="F6" s="361"/>
+      <x:c r="H6" s="448" t="n">
         <x:f>SUMIFS('Panel Data'!$L$2:$L$205,'Panel Data'!$A$2:$A$205,$D$6,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
         <x:v>39.06941683269926</x:v>
       </x:c>
-      <x:c r="I6" s="381"/>
-      <x:c r="J6" s="382"/>
-      <x:c r="K6" s="389" t="n">
+      <x:c r="I6" s="449"/>
+      <x:c r="J6" s="450"/>
+      <x:c r="K6" s="457" t="n">
         <x:f>SUMIFS('Panel Data'!$F$2:$F$205,'Panel Data'!$A$2:$A$205,$D$6,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
         <x:v>73958</x:v>
       </x:c>
-      <x:c r="L6" s="381"/>
-      <x:c r="M6" s="382"/>
+      <x:c r="L6" s="449"/>
+      <x:c r="M6" s="450"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="342"/>
-      <x:c r="B7" s="343"/>
-      <x:c r="C7" s="344"/>
-      <x:c r="D7" s="342"/>
-      <x:c r="E7" s="343"/>
-      <x:c r="F7" s="344"/>
-      <x:c r="H7" s="383"/>
-      <x:c r="I7" s="384"/>
-      <x:c r="J7" s="385"/>
-      <x:c r="K7" s="383"/>
-      <x:c r="L7" s="384"/>
-      <x:c r="M7" s="385"/>
+      <x:c r="A7" s="362"/>
+      <x:c r="B7" s="363"/>
+      <x:c r="C7" s="364"/>
+      <x:c r="D7" s="362"/>
+      <x:c r="E7" s="363"/>
+      <x:c r="F7" s="364"/>
+      <x:c r="H7" s="451"/>
+      <x:c r="I7" s="452"/>
+      <x:c r="J7" s="453"/>
+      <x:c r="K7" s="451"/>
+      <x:c r="L7" s="452"/>
+      <x:c r="M7" s="453"/>
     </x:row>
     <x:row r="9">
-      <x:c r="H9" s="365" t="str">
+      <x:c r="H9" s="433" t="str">
         <x:v>PROFILE QUADRANT</x:v>
       </x:c>
-      <x:c r="I9" s="365"/>
-      <x:c r="J9" s="365"/>
+      <x:c r="I9" s="433"/>
+      <x:c r="J9" s="433"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="390" t="str">
+      <x:c r="A10" s="458" t="str">
         <x:v>Economic dimension</x:v>
       </x:c>
-      <x:c r="B10" s="390" t="str">
+      <x:c r="B10" s="458" t="str">
         <x:v>Selected value</x:v>
       </x:c>
-      <x:c r="C10" s="390" t="str">
+      <x:c r="C10" s="458" t="str">
         <x:v>Percentile</x:v>
       </x:c>
-      <x:c r="D10" s="390" t="str">
+      <x:c r="D10" s="458" t="str">
         <x:v>Interpretation</x:v>
       </x:c>
-      <x:c r="E10" s="390" t="str">
+      <x:c r="E10" s="458" t="str">
         <x:v>Rank / 51</x:v>
       </x:c>
-      <x:c r="H10" s="418" t="str">
+      <x:c r="H10" s="486" t="str">
         <x:f>IF(C11&gt;=0.5,IF(C12&gt;=0.5,"HIGH EXPOSURE / HIGH SEVERITY","HIGH EXPOSURE / LOWER SEVERITY"),IF(C12&gt;=0.5,"LOWER EXPOSURE / HIGH SEVERITY","LOWER EXPOSURE / LOWER SEVERITY"))</x:f>
         <x:v>LOWER EXPOSURE / LOWER SEVERITY</x:v>
       </x:c>
-      <x:c r="I10" s="419"/>
-      <x:c r="J10" s="419"/>
-      <x:c r="K10" s="419"/>
-      <x:c r="L10" s="419"/>
-      <x:c r="M10" s="420"/>
+      <x:c r="I10" s="487"/>
+      <x:c r="J10" s="487"/>
+      <x:c r="K10" s="487"/>
+      <x:c r="L10" s="487"/>
+      <x:c r="M10" s="488"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
@@ -5247,12 +5563,12 @@
         <x:f>1+COUNTIFS('Panel Data'!$A$2:$A$205,$D$6,'Panel Data'!$K$2:$K$205,"&gt;"&amp;B11)</x:f>
         <x:v>31</x:v>
       </x:c>
-      <x:c r="H11" s="421"/>
-      <x:c r="I11" s="422"/>
-      <x:c r="J11" s="422"/>
-      <x:c r="K11" s="422"/>
-      <x:c r="L11" s="422"/>
-      <x:c r="M11" s="423"/>
+      <x:c r="H11" s="489"/>
+      <x:c r="I11" s="490"/>
+      <x:c r="J11" s="490"/>
+      <x:c r="K11" s="490"/>
+      <x:c r="L11" s="490"/>
+      <x:c r="M11" s="491"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
@@ -5274,12 +5590,12 @@
         <x:f>1+COUNTIFS('Panel Data'!$A$2:$A$205,$D$6,'Panel Data'!$M$2:$M$205,"&gt;"&amp;B12)</x:f>
         <x:v>37</x:v>
       </x:c>
-      <x:c r="H12" s="424"/>
-      <x:c r="I12" s="425"/>
-      <x:c r="J12" s="425"/>
-      <x:c r="K12" s="425"/>
-      <x:c r="L12" s="425"/>
-      <x:c r="M12" s="426"/>
+      <x:c r="H12" s="492"/>
+      <x:c r="I12" s="493"/>
+      <x:c r="J12" s="493"/>
+      <x:c r="K12" s="493"/>
+      <x:c r="L12" s="493"/>
+      <x:c r="M12" s="494"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
@@ -5395,108 +5711,108 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="445" t="str">
+      <x:c r="A24" s="513" t="str">
         <x:v>ECONOMIC READING
 Exposure measures how often residents report fraud; severity measures the average dollars lost per complaint. The quadrant prevents a single ranking from hiding the mechanism. A state can experience high total harm because exposure is elevated, losses are severe, or both.</x:v>
       </x:c>
-      <x:c r="B24" s="446"/>
-      <x:c r="C24" s="446"/>
-      <x:c r="D24" s="446"/>
-      <x:c r="E24" s="447"/>
+      <x:c r="B24" s="514"/>
+      <x:c r="C24" s="514"/>
+      <x:c r="D24" s="514"/>
+      <x:c r="E24" s="515"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="448"/>
-      <x:c r="B25" s="449"/>
-      <x:c r="C25" s="449"/>
-      <x:c r="D25" s="449"/>
-      <x:c r="E25" s="450"/>
+      <x:c r="A25" s="516"/>
+      <x:c r="B25" s="517"/>
+      <x:c r="C25" s="517"/>
+      <x:c r="D25" s="517"/>
+      <x:c r="E25" s="518"/>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="448"/>
-      <x:c r="B26" s="449"/>
-      <x:c r="C26" s="449"/>
-      <x:c r="D26" s="449"/>
-      <x:c r="E26" s="450"/>
+      <x:c r="A26" s="516"/>
+      <x:c r="B26" s="517"/>
+      <x:c r="C26" s="517"/>
+      <x:c r="D26" s="517"/>
+      <x:c r="E26" s="518"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="448"/>
-      <x:c r="B27" s="449"/>
-      <x:c r="C27" s="449"/>
-      <x:c r="D27" s="449"/>
-      <x:c r="E27" s="450"/>
+      <x:c r="A27" s="516"/>
+      <x:c r="B27" s="517"/>
+      <x:c r="C27" s="517"/>
+      <x:c r="D27" s="517"/>
+      <x:c r="E27" s="518"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="451"/>
-      <x:c r="B28" s="452"/>
-      <x:c r="C28" s="452"/>
-      <x:c r="D28" s="452"/>
-      <x:c r="E28" s="453"/>
+      <x:c r="A28" s="519"/>
+      <x:c r="B28" s="520"/>
+      <x:c r="C28" s="520"/>
+      <x:c r="D28" s="520"/>
+      <x:c r="E28" s="521"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="456" t="str">
+      <x:c r="A31" s="524" t="str">
         <x:v>CHALLENGE: Find one state with high exposure but lower severity, then another with lower exposure but high severity. What different prevention strategies might each profile suggest?</x:v>
       </x:c>
-      <x:c r="B31" s="456"/>
-      <x:c r="C31" s="456"/>
-      <x:c r="D31" s="456"/>
-      <x:c r="E31" s="456"/>
-      <x:c r="F31" s="456"/>
-      <x:c r="G31" s="456"/>
-      <x:c r="H31" s="456"/>
-      <x:c r="I31" s="456"/>
-      <x:c r="J31" s="456"/>
-      <x:c r="K31" s="456"/>
-      <x:c r="L31" s="456"/>
-      <x:c r="M31" s="456"/>
-      <x:c r="N31" s="456"/>
+      <x:c r="B31" s="524"/>
+      <x:c r="C31" s="524"/>
+      <x:c r="D31" s="524"/>
+      <x:c r="E31" s="524"/>
+      <x:c r="F31" s="524"/>
+      <x:c r="G31" s="524"/>
+      <x:c r="H31" s="524"/>
+      <x:c r="I31" s="524"/>
+      <x:c r="J31" s="524"/>
+      <x:c r="K31" s="524"/>
+      <x:c r="L31" s="524"/>
+      <x:c r="M31" s="524"/>
+      <x:c r="N31" s="524"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="456"/>
-      <x:c r="B32" s="456"/>
-      <x:c r="C32" s="456"/>
-      <x:c r="D32" s="456"/>
-      <x:c r="E32" s="456"/>
-      <x:c r="F32" s="456"/>
-      <x:c r="G32" s="456"/>
-      <x:c r="H32" s="456"/>
-      <x:c r="I32" s="456"/>
-      <x:c r="J32" s="456"/>
-      <x:c r="K32" s="456"/>
-      <x:c r="L32" s="456"/>
-      <x:c r="M32" s="456"/>
-      <x:c r="N32" s="456"/>
+      <x:c r="A32" s="524"/>
+      <x:c r="B32" s="524"/>
+      <x:c r="C32" s="524"/>
+      <x:c r="D32" s="524"/>
+      <x:c r="E32" s="524"/>
+      <x:c r="F32" s="524"/>
+      <x:c r="G32" s="524"/>
+      <x:c r="H32" s="524"/>
+      <x:c r="I32" s="524"/>
+      <x:c r="J32" s="524"/>
+      <x:c r="K32" s="524"/>
+      <x:c r="L32" s="524"/>
+      <x:c r="M32" s="524"/>
+      <x:c r="N32" s="524"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="456"/>
-      <x:c r="B33" s="456"/>
-      <x:c r="C33" s="456"/>
-      <x:c r="D33" s="456"/>
-      <x:c r="E33" s="456"/>
-      <x:c r="F33" s="456"/>
-      <x:c r="G33" s="456"/>
-      <x:c r="H33" s="456"/>
-      <x:c r="I33" s="456"/>
-      <x:c r="J33" s="456"/>
-      <x:c r="K33" s="456"/>
-      <x:c r="L33" s="456"/>
-      <x:c r="M33" s="456"/>
-      <x:c r="N33" s="456"/>
+      <x:c r="A33" s="524"/>
+      <x:c r="B33" s="524"/>
+      <x:c r="C33" s="524"/>
+      <x:c r="D33" s="524"/>
+      <x:c r="E33" s="524"/>
+      <x:c r="F33" s="524"/>
+      <x:c r="G33" s="524"/>
+      <x:c r="H33" s="524"/>
+      <x:c r="I33" s="524"/>
+      <x:c r="J33" s="524"/>
+      <x:c r="K33" s="524"/>
+      <x:c r="L33" s="524"/>
+      <x:c r="M33" s="524"/>
+      <x:c r="N33" s="524"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="456"/>
-      <x:c r="B34" s="456"/>
-      <x:c r="C34" s="456"/>
-      <x:c r="D34" s="456"/>
-      <x:c r="E34" s="456"/>
-      <x:c r="F34" s="456"/>
-      <x:c r="G34" s="456"/>
-      <x:c r="H34" s="456"/>
-      <x:c r="I34" s="456"/>
-      <x:c r="J34" s="456"/>
-      <x:c r="K34" s="456"/>
-      <x:c r="L34" s="456"/>
-      <x:c r="M34" s="456"/>
-      <x:c r="N34" s="456"/>
+      <x:c r="A34" s="524"/>
+      <x:c r="B34" s="524"/>
+      <x:c r="C34" s="524"/>
+      <x:c r="D34" s="524"/>
+      <x:c r="E34" s="524"/>
+      <x:c r="F34" s="524"/>
+      <x:c r="G34" s="524"/>
+      <x:c r="H34" s="524"/>
+      <x:c r="I34" s="524"/>
+      <x:c r="J34" s="524"/>
+      <x:c r="K34" s="524"/>
+      <x:c r="L34" s="524"/>
+      <x:c r="M34" s="524"/>
+      <x:c r="N34" s="524"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5516,8 +5832,13 @@
     <x:mergeCell ref="A24:E28"/>
     <x:mergeCell ref="A31:N34"/>
   </x:mergeCells>
+  <x:conditionalFormatting sqref="D11:D13">
+    <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="High"/>
+    <x:cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="Middle"/>
+    <x:cfRule type="containsText" dxfId="4" priority="3" operator="containsText" text="Low"/>
+  </x:conditionalFormatting>
   <x:conditionalFormatting sqref="C11:C13">
-    <x:cfRule type="dataBar" priority="1">
+    <x:cfRule type="dataBar" priority="4">
       <x:dataBar>
         <x:cfvo type="min"/>
         <x:cfvo type="max"/>
@@ -5525,10 +5846,16 @@
       </x:dataBar>
       <x:extLst>
         <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{145E6682-420D-8C48-59AD-7E3EAA9F4932}</x14:id>
+          <x14:id>{F4EA9E46-60B3-0FA8-7EE2-2627DF91B694}</x14:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="H10:M12">
+    <x:cfRule type="containsText" dxfId="5" priority="5" operator="containsText" text="HIGH EXPOSURE / HIGH SEVERITY"/>
+    <x:cfRule type="containsText" dxfId="6" priority="6" operator="containsText" text="HIGH EXPOSURE / LOWER SEVERITY"/>
+    <x:cfRule type="containsText" dxfId="7" priority="7" operator="containsText" text="LOWER EXPOSURE / HIGH SEVERITY"/>
+    <x:cfRule type="containsText" dxfId="8" priority="8" operator="containsText" text="LOWER EXPOSURE / LOWER SEVERITY"/>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="A6">
@@ -5539,12 +5866,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce81485bf7164b44"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bcd763ac4dd4232"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting>
-          <x14:cfRule type="dataBar" priority="1" id="{145E6682-420D-8C48-59AD-7E3EAA9F4932}">
+          <x14:cfRule type="dataBar" priority="4" id="{F4EA9E46-60B3-0FA8-7EE2-2627DF91B694}">
             <x14:dataBar gradient="1">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -5580,56 +5907,56 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="324" t="str">
+      <x:c r="A1" s="344" t="str">
         <x:v>SCENARIO LAB — WHAT WOULD THE MODELS IMPLY?</x:v>
       </x:c>
-      <x:c r="B1" s="324"/>
-      <x:c r="C1" s="324"/>
-      <x:c r="D1" s="324"/>
-      <x:c r="E1" s="324"/>
-      <x:c r="F1" s="324"/>
-      <x:c r="G1" s="324"/>
-      <x:c r="H1" s="324"/>
-      <x:c r="I1" s="324"/>
-      <x:c r="J1" s="324"/>
-      <x:c r="K1" s="324"/>
-      <x:c r="L1" s="324"/>
-      <x:c r="M1" s="324"/>
-      <x:c r="N1" s="324"/>
+      <x:c r="B1" s="344"/>
+      <x:c r="C1" s="344"/>
+      <x:c r="D1" s="344"/>
+      <x:c r="E1" s="344"/>
+      <x:c r="F1" s="344"/>
+      <x:c r="G1" s="344"/>
+      <x:c r="H1" s="344"/>
+      <x:c r="I1" s="344"/>
+      <x:c r="J1" s="344"/>
+      <x:c r="K1" s="344"/>
+      <x:c r="L1" s="344"/>
+      <x:c r="M1" s="344"/>
+      <x:c r="N1" s="344"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="324"/>
-      <x:c r="B2" s="324"/>
-      <x:c r="C2" s="324"/>
-      <x:c r="D2" s="324"/>
-      <x:c r="E2" s="324"/>
-      <x:c r="F2" s="324"/>
-      <x:c r="G2" s="324"/>
-      <x:c r="H2" s="324"/>
-      <x:c r="I2" s="324"/>
-      <x:c r="J2" s="324"/>
-      <x:c r="K2" s="324"/>
-      <x:c r="L2" s="324"/>
-      <x:c r="M2" s="324"/>
-      <x:c r="N2" s="324"/>
+      <x:c r="A2" s="344"/>
+      <x:c r="B2" s="344"/>
+      <x:c r="C2" s="344"/>
+      <x:c r="D2" s="344"/>
+      <x:c r="E2" s="344"/>
+      <x:c r="F2" s="344"/>
+      <x:c r="G2" s="344"/>
+      <x:c r="H2" s="344"/>
+      <x:c r="I2" s="344"/>
+      <x:c r="J2" s="344"/>
+      <x:c r="K2" s="344"/>
+      <x:c r="L2" s="344"/>
+      <x:c r="M2" s="344"/>
+      <x:c r="N2" s="344"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="354" t="str">
+      <x:c r="A3" s="422" t="str">
         <x:v>Choose a state, year, and hypothetical income change. The workbook translates each estimated elasticity into a model-implied loss-per-person scenario.</x:v>
       </x:c>
-      <x:c r="B3" s="354"/>
-      <x:c r="C3" s="354"/>
-      <x:c r="D3" s="354"/>
-      <x:c r="E3" s="354"/>
-      <x:c r="F3" s="354"/>
-      <x:c r="G3" s="354"/>
-      <x:c r="H3" s="354"/>
-      <x:c r="I3" s="354"/>
-      <x:c r="J3" s="354"/>
-      <x:c r="K3" s="354"/>
-      <x:c r="L3" s="354"/>
-      <x:c r="M3" s="354"/>
-      <x:c r="N3" s="354"/>
+      <x:c r="B3" s="422"/>
+      <x:c r="C3" s="422"/>
+      <x:c r="D3" s="422"/>
+      <x:c r="E3" s="422"/>
+      <x:c r="F3" s="422"/>
+      <x:c r="G3" s="422"/>
+      <x:c r="H3" s="422"/>
+      <x:c r="I3" s="422"/>
+      <x:c r="J3" s="422"/>
+      <x:c r="K3" s="422"/>
+      <x:c r="L3" s="422"/>
+      <x:c r="M3" s="422"/>
+      <x:c r="N3" s="422"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="68" t="str">
@@ -5655,21 +5982,21 @@
       <x:c r="N5" s="37"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="339" t="str">
+      <x:c r="A6" s="359" t="str">
         <x:v>North Carolina</x:v>
       </x:c>
-      <x:c r="B6" s="340"/>
-      <x:c r="C6" s="341"/>
-      <x:c r="D6" s="339" t="n">
+      <x:c r="B6" s="360"/>
+      <x:c r="C6" s="361"/>
+      <x:c r="D6" s="359" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="E6" s="340"/>
-      <x:c r="F6" s="341"/>
-      <x:c r="G6" s="355" t="n">
+      <x:c r="E6" s="360"/>
+      <x:c r="F6" s="361"/>
+      <x:c r="G6" s="423" t="n">
         <x:v>0.1</x:v>
       </x:c>
-      <x:c r="H6" s="340"/>
-      <x:c r="I6" s="341"/>
+      <x:c r="H6" s="360"/>
+      <x:c r="I6" s="361"/>
       <x:c r="K6" s="316" t="str">
         <x:v>Median income</x:v>
       </x:c>
@@ -5678,20 +6005,20 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="342"/>
-      <x:c r="B7" s="343"/>
-      <x:c r="C7" s="344"/>
-      <x:c r="D7" s="342"/>
-      <x:c r="E7" s="343"/>
-      <x:c r="F7" s="344"/>
-      <x:c r="G7" s="342"/>
-      <x:c r="H7" s="343"/>
-      <x:c r="I7" s="344"/>
-      <x:c r="K7" s="362" t="n">
+      <x:c r="A7" s="362"/>
+      <x:c r="B7" s="363"/>
+      <x:c r="C7" s="364"/>
+      <x:c r="D7" s="362"/>
+      <x:c r="E7" s="363"/>
+      <x:c r="F7" s="364"/>
+      <x:c r="G7" s="362"/>
+      <x:c r="H7" s="363"/>
+      <x:c r="I7" s="364"/>
+      <x:c r="K7" s="430" t="n">
         <x:f>SUMIFS('Panel Data'!$F$2:$F$205,'Panel Data'!$A$2:$A$205,$D$6,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
         <x:v>73958</x:v>
       </x:c>
-      <x:c r="L7" s="363" t="n">
+      <x:c r="L7" s="431" t="n">
         <x:f>SUMIFS('Panel Data'!$L$2:$L$205,'Panel Data'!$A$2:$A$205,$D$6,'Panel Data'!$B$2:$B$205,$A$6)</x:f>
         <x:v>39.06941683269926</x:v>
       </x:c>
@@ -5740,7 +6067,7 @@
         <x:f>C12*(1+$G$6)^B12</x:f>
         <x:v>45.297932070756154</x:v>
       </x:c>
-      <x:c r="E12" s="364" t="n">
+      <x:c r="E12" s="432" t="n">
         <x:f>D12/C12-1</x:f>
         <x:v>0.15942176113680606</x:v>
       </x:c>
@@ -5760,7 +6087,7 @@
         <x:f>C13*(1+$G$6)^B13</x:f>
         <x:v>48.12869920014451</x:v>
       </x:c>
-      <x:c r="E13" s="364" t="n">
+      <x:c r="E13" s="432" t="n">
         <x:f>D13/C13-1</x:f>
         <x:v>0.23187657000969253</x:v>
       </x:c>
@@ -5780,7 +6107,7 @@
         <x:f>C14*(1+$G$6)^B14</x:f>
         <x:v>42.51598454771643</x:v>
       </x:c>
-      <x:c r="E14" s="364" t="n">
+      <x:c r="E14" s="432" t="n">
         <x:f>D14/C14-1</x:f>
         <x:v>0.0882165129255923</x:v>
       </x:c>
@@ -5847,137 +6174,137 @@
       <x:c r="E24" s="168"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="349" t="str">
+      <x:c r="A27" s="389" t="str">
         <x:v>IMPORTANT: THIS IS NOT A CAUSAL FORECAST
 The elasticities describe associations in state-level data. Changing income alone would not mechanically cause the displayed change in fraud loss. Reporting behavior, target value, internet exposure, enforcement, and omitted state characteristics may all contribute. Use this lab to study sensitivity and identification—not to predict policy effects.</x:v>
       </x:c>
-      <x:c r="B27" s="349"/>
-      <x:c r="C27" s="349"/>
-      <x:c r="D27" s="349"/>
-      <x:c r="E27" s="349"/>
-      <x:c r="F27" s="349"/>
-      <x:c r="G27" s="349"/>
-      <x:c r="H27" s="349"/>
-      <x:c r="I27" s="349"/>
-      <x:c r="J27" s="349"/>
-      <x:c r="K27" s="349"/>
-      <x:c r="L27" s="349"/>
-      <x:c r="M27" s="349"/>
-      <x:c r="N27" s="349"/>
+      <x:c r="B27" s="389"/>
+      <x:c r="C27" s="389"/>
+      <x:c r="D27" s="389"/>
+      <x:c r="E27" s="389"/>
+      <x:c r="F27" s="389"/>
+      <x:c r="G27" s="389"/>
+      <x:c r="H27" s="389"/>
+      <x:c r="I27" s="389"/>
+      <x:c r="J27" s="389"/>
+      <x:c r="K27" s="389"/>
+      <x:c r="L27" s="389"/>
+      <x:c r="M27" s="389"/>
+      <x:c r="N27" s="389"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="349"/>
-      <x:c r="B28" s="349"/>
-      <x:c r="C28" s="349"/>
-      <x:c r="D28" s="349"/>
-      <x:c r="E28" s="349"/>
-      <x:c r="F28" s="349"/>
-      <x:c r="G28" s="349"/>
-      <x:c r="H28" s="349"/>
-      <x:c r="I28" s="349"/>
-      <x:c r="J28" s="349"/>
-      <x:c r="K28" s="349"/>
-      <x:c r="L28" s="349"/>
-      <x:c r="M28" s="349"/>
-      <x:c r="N28" s="349"/>
+      <x:c r="A28" s="389"/>
+      <x:c r="B28" s="389"/>
+      <x:c r="C28" s="389"/>
+      <x:c r="D28" s="389"/>
+      <x:c r="E28" s="389"/>
+      <x:c r="F28" s="389"/>
+      <x:c r="G28" s="389"/>
+      <x:c r="H28" s="389"/>
+      <x:c r="I28" s="389"/>
+      <x:c r="J28" s="389"/>
+      <x:c r="K28" s="389"/>
+      <x:c r="L28" s="389"/>
+      <x:c r="M28" s="389"/>
+      <x:c r="N28" s="389"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="349"/>
-      <x:c r="B29" s="349"/>
-      <x:c r="C29" s="349"/>
-      <x:c r="D29" s="349"/>
-      <x:c r="E29" s="349"/>
-      <x:c r="F29" s="349"/>
-      <x:c r="G29" s="349"/>
-      <x:c r="H29" s="349"/>
-      <x:c r="I29" s="349"/>
-      <x:c r="J29" s="349"/>
-      <x:c r="K29" s="349"/>
-      <x:c r="L29" s="349"/>
-      <x:c r="M29" s="349"/>
-      <x:c r="N29" s="349"/>
+      <x:c r="A29" s="389"/>
+      <x:c r="B29" s="389"/>
+      <x:c r="C29" s="389"/>
+      <x:c r="D29" s="389"/>
+      <x:c r="E29" s="389"/>
+      <x:c r="F29" s="389"/>
+      <x:c r="G29" s="389"/>
+      <x:c r="H29" s="389"/>
+      <x:c r="I29" s="389"/>
+      <x:c r="J29" s="389"/>
+      <x:c r="K29" s="389"/>
+      <x:c r="L29" s="389"/>
+      <x:c r="M29" s="389"/>
+      <x:c r="N29" s="389"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="349"/>
-      <x:c r="B30" s="349"/>
-      <x:c r="C30" s="349"/>
-      <x:c r="D30" s="349"/>
-      <x:c r="E30" s="349"/>
-      <x:c r="F30" s="349"/>
-      <x:c r="G30" s="349"/>
-      <x:c r="H30" s="349"/>
-      <x:c r="I30" s="349"/>
-      <x:c r="J30" s="349"/>
-      <x:c r="K30" s="349"/>
-      <x:c r="L30" s="349"/>
-      <x:c r="M30" s="349"/>
-      <x:c r="N30" s="349"/>
+      <x:c r="A30" s="389"/>
+      <x:c r="B30" s="389"/>
+      <x:c r="C30" s="389"/>
+      <x:c r="D30" s="389"/>
+      <x:c r="E30" s="389"/>
+      <x:c r="F30" s="389"/>
+      <x:c r="G30" s="389"/>
+      <x:c r="H30" s="389"/>
+      <x:c r="I30" s="389"/>
+      <x:c r="J30" s="389"/>
+      <x:c r="K30" s="389"/>
+      <x:c r="L30" s="389"/>
+      <x:c r="M30" s="389"/>
+      <x:c r="N30" s="389"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="349"/>
-      <x:c r="B31" s="349"/>
-      <x:c r="C31" s="349"/>
-      <x:c r="D31" s="349"/>
-      <x:c r="E31" s="349"/>
-      <x:c r="F31" s="349"/>
-      <x:c r="G31" s="349"/>
-      <x:c r="H31" s="349"/>
-      <x:c r="I31" s="349"/>
-      <x:c r="J31" s="349"/>
-      <x:c r="K31" s="349"/>
-      <x:c r="L31" s="349"/>
-      <x:c r="M31" s="349"/>
-      <x:c r="N31" s="349"/>
+      <x:c r="A31" s="389"/>
+      <x:c r="B31" s="389"/>
+      <x:c r="C31" s="389"/>
+      <x:c r="D31" s="389"/>
+      <x:c r="E31" s="389"/>
+      <x:c r="F31" s="389"/>
+      <x:c r="G31" s="389"/>
+      <x:c r="H31" s="389"/>
+      <x:c r="I31" s="389"/>
+      <x:c r="J31" s="389"/>
+      <x:c r="K31" s="389"/>
+      <x:c r="L31" s="389"/>
+      <x:c r="M31" s="389"/>
+      <x:c r="N31" s="389"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="354" t="str">
+      <x:c r="A33" s="422" t="str">
         <x:v>CHALLENGE: Set income change to +10%. Which specification produces the smallest implied change? Why might the fixed-effects estimate be less precise even though its point estimate is larger?</x:v>
       </x:c>
-      <x:c r="B33" s="354"/>
-      <x:c r="C33" s="354"/>
-      <x:c r="D33" s="354"/>
-      <x:c r="E33" s="354"/>
-      <x:c r="F33" s="354"/>
-      <x:c r="G33" s="354"/>
-      <x:c r="H33" s="354"/>
-      <x:c r="I33" s="354"/>
-      <x:c r="J33" s="354"/>
-      <x:c r="K33" s="354"/>
-      <x:c r="L33" s="354"/>
-      <x:c r="M33" s="354"/>
-      <x:c r="N33" s="354"/>
+      <x:c r="B33" s="422"/>
+      <x:c r="C33" s="422"/>
+      <x:c r="D33" s="422"/>
+      <x:c r="E33" s="422"/>
+      <x:c r="F33" s="422"/>
+      <x:c r="G33" s="422"/>
+      <x:c r="H33" s="422"/>
+      <x:c r="I33" s="422"/>
+      <x:c r="J33" s="422"/>
+      <x:c r="K33" s="422"/>
+      <x:c r="L33" s="422"/>
+      <x:c r="M33" s="422"/>
+      <x:c r="N33" s="422"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="354"/>
-      <x:c r="B34" s="354"/>
-      <x:c r="C34" s="354"/>
-      <x:c r="D34" s="354"/>
-      <x:c r="E34" s="354"/>
-      <x:c r="F34" s="354"/>
-      <x:c r="G34" s="354"/>
-      <x:c r="H34" s="354"/>
-      <x:c r="I34" s="354"/>
-      <x:c r="J34" s="354"/>
-      <x:c r="K34" s="354"/>
-      <x:c r="L34" s="354"/>
-      <x:c r="M34" s="354"/>
-      <x:c r="N34" s="354"/>
+      <x:c r="A34" s="422"/>
+      <x:c r="B34" s="422"/>
+      <x:c r="C34" s="422"/>
+      <x:c r="D34" s="422"/>
+      <x:c r="E34" s="422"/>
+      <x:c r="F34" s="422"/>
+      <x:c r="G34" s="422"/>
+      <x:c r="H34" s="422"/>
+      <x:c r="I34" s="422"/>
+      <x:c r="J34" s="422"/>
+      <x:c r="K34" s="422"/>
+      <x:c r="L34" s="422"/>
+      <x:c r="M34" s="422"/>
+      <x:c r="N34" s="422"/>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="354"/>
-      <x:c r="B35" s="354"/>
-      <x:c r="C35" s="354"/>
-      <x:c r="D35" s="354"/>
-      <x:c r="E35" s="354"/>
-      <x:c r="F35" s="354"/>
-      <x:c r="G35" s="354"/>
-      <x:c r="H35" s="354"/>
-      <x:c r="I35" s="354"/>
-      <x:c r="J35" s="354"/>
-      <x:c r="K35" s="354"/>
-      <x:c r="L35" s="354"/>
-      <x:c r="M35" s="354"/>
-      <x:c r="N35" s="354"/>
+      <x:c r="A35" s="422"/>
+      <x:c r="B35" s="422"/>
+      <x:c r="C35" s="422"/>
+      <x:c r="D35" s="422"/>
+      <x:c r="E35" s="422"/>
+      <x:c r="F35" s="422"/>
+      <x:c r="G35" s="422"/>
+      <x:c r="H35" s="422"/>
+      <x:c r="I35" s="422"/>
+      <x:c r="J35" s="422"/>
+      <x:c r="K35" s="422"/>
+      <x:c r="L35" s="422"/>
+      <x:c r="M35" s="422"/>
+      <x:c r="N35" s="422"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6023,7 +6350,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a2c722445934657"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb6b7b7de05d4292"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -6451,7 +6778,7 @@
     <x:mergeCell ref="A40:N42"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R685c14d942a84026"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80b308999e4840e6"/>
 </x:worksheet>
 </file>
 
@@ -6861,94 +7188,114 @@
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="257" t="str">
-        <x:v>Identification verdict: adding years improves power and lets the project separate permanent geographic differences from changes within a state. The fixed-effects model does not confirm a causal income effect, so the paper treats income as a marker of target value and correlated state characteristics.</x:v>
-      </x:c>
-      <x:c r="B30" s="257"/>
-      <x:c r="C30" s="257"/>
-      <x:c r="D30" s="257"/>
-      <x:c r="E30" s="257"/>
-      <x:c r="F30" s="257"/>
-      <x:c r="G30" s="257"/>
-      <x:c r="H30" s="257" t="n">
+      <x:c r="H30" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="I30" s="257" t="str">
+      <x:c r="I30" t="str">
         <x:v>Midwest</x:v>
       </x:c>
-      <x:c r="J30" s="322" t="n">
+      <x:c r="J30" s="225" t="n">
         <x:v>38.10106403927721</x:v>
       </x:c>
-      <x:c r="K30" s="257"/>
-      <x:c r="L30" s="257"/>
-      <x:c r="M30" s="257"/>
-      <x:c r="N30" s="257"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="257"/>
-      <x:c r="B31" s="257"/>
-      <x:c r="C31" s="257"/>
-      <x:c r="D31" s="257"/>
-      <x:c r="E31" s="257"/>
-      <x:c r="F31" s="257"/>
-      <x:c r="G31" s="257"/>
-      <x:c r="H31" s="257" t="n">
+      <x:c r="H31" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="I31" s="257" t="str">
+      <x:c r="I31" t="str">
         <x:v>Northeast</x:v>
       </x:c>
-      <x:c r="J31" s="322" t="n">
+      <x:c r="J31" s="225" t="n">
         <x:v>56.52968852436764</x:v>
       </x:c>
-      <x:c r="K31" s="257"/>
-      <x:c r="L31" s="257"/>
-      <x:c r="M31" s="257"/>
-      <x:c r="N31" s="257"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="257"/>
-      <x:c r="B32" s="257"/>
-      <x:c r="C32" s="257"/>
-      <x:c r="D32" s="257"/>
-      <x:c r="E32" s="257"/>
-      <x:c r="F32" s="257"/>
-      <x:c r="G32" s="257"/>
-      <x:c r="H32" s="257" t="n">
+      <x:c r="H32" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="I32" s="257" t="str">
+      <x:c r="I32" t="str">
         <x:v>South</x:v>
       </x:c>
-      <x:c r="J32" s="322" t="n">
+      <x:c r="J32" s="225" t="n">
         <x:v>50.83281948408471</x:v>
       </x:c>
-      <x:c r="K32" s="257"/>
-      <x:c r="L32" s="257"/>
-      <x:c r="M32" s="257"/>
-      <x:c r="N32" s="257"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="257"/>
-      <x:c r="B33" s="257"/>
-      <x:c r="C33" s="257"/>
-      <x:c r="D33" s="257"/>
-      <x:c r="E33" s="257"/>
-      <x:c r="F33" s="257"/>
-      <x:c r="G33" s="257"/>
-      <x:c r="H33" s="257" t="n">
+      <x:c r="H33" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="I33" s="257" t="str">
+      <x:c r="I33" t="str">
         <x:v>West</x:v>
       </x:c>
-      <x:c r="J33" s="322" t="n">
+      <x:c r="J33" s="225" t="n">
         <x:v>77.59990114199603</x:v>
       </x:c>
-      <x:c r="K33" s="257"/>
-      <x:c r="L33" s="257"/>
-      <x:c r="M33" s="257"/>
-      <x:c r="N33" s="257"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="335" t="str">
+        <x:v>Identification verdict: adding years improves power and lets the project separate permanent geographic differences from changes within a state. The fixed-effects model does not confirm a causal income effect, so the project treats income as a marker of target value and correlated state characteristics.</x:v>
+      </x:c>
+      <x:c r="B35" s="336"/>
+      <x:c r="C35" s="336"/>
+      <x:c r="D35" s="336"/>
+      <x:c r="E35" s="336"/>
+      <x:c r="F35" s="336"/>
+      <x:c r="G35" s="336"/>
+      <x:c r="H35" s="336"/>
+      <x:c r="I35" s="336"/>
+      <x:c r="J35" s="336"/>
+      <x:c r="K35" s="336"/>
+      <x:c r="L35" s="336"/>
+      <x:c r="M35" s="336"/>
+      <x:c r="N35" s="337"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="338"/>
+      <x:c r="B36" s="257"/>
+      <x:c r="C36" s="257"/>
+      <x:c r="D36" s="257"/>
+      <x:c r="E36" s="257"/>
+      <x:c r="F36" s="257"/>
+      <x:c r="G36" s="257"/>
+      <x:c r="H36" s="257"/>
+      <x:c r="I36" s="257"/>
+      <x:c r="J36" s="257"/>
+      <x:c r="K36" s="257"/>
+      <x:c r="L36" s="257"/>
+      <x:c r="M36" s="257"/>
+      <x:c r="N36" s="339"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="338"/>
+      <x:c r="B37" s="257"/>
+      <x:c r="C37" s="257"/>
+      <x:c r="D37" s="257"/>
+      <x:c r="E37" s="257"/>
+      <x:c r="F37" s="257"/>
+      <x:c r="G37" s="257"/>
+      <x:c r="H37" s="257"/>
+      <x:c r="I37" s="257"/>
+      <x:c r="J37" s="257"/>
+      <x:c r="K37" s="257"/>
+      <x:c r="L37" s="257"/>
+      <x:c r="M37" s="257"/>
+      <x:c r="N37" s="339"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="340"/>
+      <x:c r="B38" s="341"/>
+      <x:c r="C38" s="341"/>
+      <x:c r="D38" s="341"/>
+      <x:c r="E38" s="341"/>
+      <x:c r="F38" s="341"/>
+      <x:c r="G38" s="341"/>
+      <x:c r="H38" s="341"/>
+      <x:c r="I38" s="341"/>
+      <x:c r="J38" s="341"/>
+      <x:c r="K38" s="341"/>
+      <x:c r="L38" s="341"/>
+      <x:c r="M38" s="341"/>
+      <x:c r="N38" s="342"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6958,10 +7305,10 @@
     <x:mergeCell ref="H5:N5"/>
     <x:mergeCell ref="H6:N14"/>
     <x:mergeCell ref="H16:N16"/>
-    <x:mergeCell ref="A30:N33"/>
+    <x:mergeCell ref="A35:N38"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1b5b7e860cb4a52"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2499f5b385946bb"/>
 </x:worksheet>
 </file>
 
@@ -10065,7 +10412,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8da9eb0600c412b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6820dcbb3cf147bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20341,7 +20688,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64c5bc17a1cb4665"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cee8195a76a4f5e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20758,7 +21105,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7c59e62c9324a73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc19f8e4bfe84828"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Correct internet-crime terminology and refresh verified workbook previews
</commit_message>
<xml_diff>
--- a/Scam_Geography_Interactive_Economics_Project.xlsx
+++ b/Scam_Geography_Interactive_Economics_Project.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Re3267b9c02d2469a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interactive Econ Lab" sheetId="2" r:id="R81995f3df5a14089"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Scorecard" sheetId="3" r:id="Rd570963bebc843f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Lab" sheetId="4" r:id="R60ea0c275cab4988"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" r:id="R6dc29620f4814471"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Dashboard" sheetId="6" r:id="R1eb387e44e1d42e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Data" sheetId="7" r:id="R77f616f387e8481f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Data" sheetId="8" r:id="R54ed324b5d2047be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression" sheetId="9" r:id="Rb30f5e8f3d494ff5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Models" sheetId="10" r:id="R349598b681fe4031"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Notes" sheetId="11" r:id="R1d10a625128340a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart Data" sheetId="12" r:id="R1d253b4704784fbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R32a39f204f664b7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interactive Econ Lab" sheetId="2" r:id="R74468ba5292b45dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Scorecard" sheetId="3" r:id="Rb8a0ef54ebb54a97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Lab" sheetId="4" r:id="R6bc73e1784564986"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" r:id="R6c1b97d3e84d434e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Dashboard" sheetId="6" r:id="R1937eb13d0434ae6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Data" sheetId="7" r:id="R17d3adb11b0f42ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Data" sheetId="8" r:id="R793aa98d4ae24e08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression" sheetId="9" r:id="R994fb3e01e184bf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel Models" sheetId="10" r:id="Ref68c4bf5ba44d82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Notes" sheetId="11" r:id="R843371a577f6464d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart Data" sheetId="12" r:id="Rb52d8406d41945ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2574,7 +2574,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R432b1023d8e74f7a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R83715f6437264a7a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2609,7 +2609,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R929337fa44844875"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra081a2ac7bb5445f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2644,7 +2644,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3c6d0db1a44647dd"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2725bf1afdd346a6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2679,7 +2679,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6e25043340ae4e1b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra03b608d72a74884"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2709,7 +2709,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R342b0701f4ce46b1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7baba1be31a34a31"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2744,7 +2744,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R857b8bcf8a8543f2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2dcf1d45f738484a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3112,7 +3112,7 @@
     <x:row r="6">
       <x:c r="A6" s="26" t="str">
         <x:v>RESEARCH QUESTION
-Where does reported online fraud impose the greatest economic harm—and do income, internet access, and demographic differences help explain the geography?</x:v>
+Where are reported internet-crime losses highest per resident, and how are they associated with income, internet access, and age structure?</x:v>
       </x:c>
       <x:c r="B6" s="27"/>
       <x:c r="C6" s="27"/>
@@ -3141,7 +3141,7 @@
       <x:c r="I7" s="31"/>
       <x:c r="K7" s="57" t="str">
         <x:v>1. Compare states in Interactive Econ Lab
-2. Diagnose mechanisms in State Scorecard
+2. Compare exposure and severity in State Scorecard
 3. Stress-test assumptions in Scenario Lab
 4. Review the panel evidence
 5. Audit Sources &amp; Notes</x:v>
@@ -3293,7 +3293,7 @@
     <x:row r="18">
       <x:c r="A18" s="132" t="str">
         <x:v>LOSS PER PERSON = COMPLAINTS PER PERSON × LOSS PER COMPLAINT
-This decomposition separates reported exposure from loss severity. A state can rank highly because more residents report fraud, because each complaint is costlier, or both.</x:v>
+This decomposition separates reported exposure from loss severity. A state can rank highly because more complaints are reported per resident, because each complaint is costlier, or both.</x:v>
       </x:c>
       <x:c r="B18" s="133"/>
       <x:c r="C18" s="133"/>
@@ -3391,7 +3391,7 @@
     <x:row r="25">
       <x:c r="A25" s="171" t="str">
         <x:v>BOTTOM LINE
-Reported loss per person nearly doubled from 2022 to 2025. Higher-income states consistently report greater losses, but the within-state estimate is imprecise. The project therefore documents a robust geographic association—not a causal effect of income growth on fraud.</x:v>
+Reported loss per person nearly doubled from 2022 to 2025. Higher-income states tend to report greater losses, but the within-state estimate is imprecise. The project therefore documents a geographic association—not a causal effect of income growth on reported losses.</x:v>
       </x:c>
       <x:c r="B25" s="171"/>
       <x:c r="C25" s="171"/>
@@ -4054,7 +4054,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R102b0bbd7e8a4a56"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a5c856eb5464852"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4108,7 +4108,7 @@
         <x:v>https://www.ic3.gov/AnnualReport/Reports/2025_IC3Report.pdf</x:v>
       </x:c>
       <x:c r="D5" s="266" t="str">
-        <x:v>Complaint data are voluntary reports, not a prevalence survey.</x:v>
+        <x:v>All-category internet-crime totals, not a fraud-only subset. Complaints are voluntary reports, not a prevalence survey.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -4882,7 +4882,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="6" t="str">
-        <x:v>Adjust the warm input cells. Every result below updates from the 2022–2025 state panel.</x:v>
+        <x:v>Use the cream cells to select states, year, and outcome. The comparison and trend chart update with your selections.</x:v>
       </x:c>
       <x:c r="B3" s="6"/>
       <x:c r="C3" s="6"/>
@@ -4989,7 +4989,7 @@
       </x:c>
       <x:c r="H10" s="160" t="str">
         <x:v>LOSS PER PERSON = COMPLAINTS PER PERSON × LOSS PER COMPLAINT
-This identity separates exposure from severity. Use the state selectors to see whether a place ranks highly because more residents report fraud, because each complaint is costlier, or both.</x:v>
+This identity separates exposure from severity. Use the state selectors to see whether a place ranks highly because more complaints are reported per resident, because each complaint is costlier, or both.</x:v>
       </x:c>
       <x:c r="I10" s="161"/>
       <x:c r="J10" s="161"/>
@@ -5228,7 +5228,7 @@
       <x:c r="C33" s="414"/>
       <x:c r="E33" s="385" t="str">
         <x:v>ECONOMICS VERDICT
-The between-state relationship is strong and survives outlier checks. The within-state estimate is imprecise, so this project supports a geographic association—not a causal claim that rising income produces fraud losses.</x:v>
+The between-state relationship is strong and survives outlier checks. The within-state estimate is imprecise, so this project supports a geographic association—not a causal claim that rising income produces reported losses.</x:v>
       </x:c>
       <x:c r="F33" s="386"/>
       <x:c r="G33" s="386"/>
@@ -5358,7 +5358,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18bf83056d0f4542"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd90fc2847f94a04"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -5713,7 +5713,7 @@
     <x:row r="24">
       <x:c r="A24" s="513" t="str">
         <x:v>ECONOMIC READING
-Exposure measures how often residents report fraud; severity measures the average dollars lost per complaint. The quadrant prevents a single ranking from hiding the mechanism. A state can experience high total harm because exposure is elevated, losses are severe, or both.</x:v>
+Exposure measures reported complaints relative to population; severity measures the average dollars lost per complaint. The quadrant separates these two components. A state can experience high total harm because exposure is elevated, losses are severe, or both.</x:v>
       </x:c>
       <x:c r="B24" s="514"/>
       <x:c r="C24" s="514"/>
@@ -5866,7 +5866,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bcd763ac4dd4232"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rede40ab07c074dd6"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -6124,7 +6124,7 @@
     <x:row r="18">
       <x:c r="A18" s="160" t="str">
         <x:v>Elasticity translates percentage changes into model-implied outcome changes. For example, an elasticity of 1.55 means a 10% income difference is associated with roughly a 15.9% difference in loss per person using the exact power formula.
-Compare the three rows. Their spread is model uncertainty—not three competing facts.</x:v>
+Compare the three rows to see how the result depends on the model specification.</x:v>
       </x:c>
       <x:c r="B18" s="161"/>
       <x:c r="C18" s="161"/>
@@ -6176,7 +6176,7 @@
     <x:row r="27">
       <x:c r="A27" s="389" t="str">
         <x:v>IMPORTANT: THIS IS NOT A CAUSAL FORECAST
-The elasticities describe associations in state-level data. Changing income alone would not mechanically cause the displayed change in fraud loss. Reporting behavior, target value, internet exposure, enforcement, and omitted state characteristics may all contribute. Use this lab to study sensitivity and identification—not to predict policy effects.</x:v>
+The elasticities describe associations in state-level data. Changing income alone would not mechanically cause the displayed change in reported loss. Reporting behavior, target value, internet exposure, enforcement, and omitted state characteristics may all contribute. Use this lab to study sensitivity and identification—not to predict policy effects.</x:v>
       </x:c>
       <x:c r="B27" s="389"/>
       <x:c r="C27" s="389"/>
@@ -6350,7 +6350,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb6b7b7de05d4292"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R497596df27944215"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -6392,7 +6392,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="198" t="str">
-        <x:v>The Geography of Online Fraud in the United States</x:v>
+        <x:v>The Geography of Reported Internet Crime in the United States</x:v>
       </x:c>
       <x:c r="B1" s="198"/>
       <x:c r="C1" s="198"/>
@@ -6778,7 +6778,7 @@
     <x:mergeCell ref="A40:N42"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80b308999e4840e6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41859c18b3264052"/>
 </x:worksheet>
 </file>
 
@@ -6804,7 +6804,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="198" t="str">
-        <x:v>Next-level evidence: four-year state panel</x:v>
+        <x:v>Reported internet crime: four-year state panel</x:v>
       </x:c>
       <x:c r="B1" s="198"/>
       <x:c r="C1" s="198"/>
@@ -6863,7 +6863,7 @@
       <x:c r="D5" s="222"/>
       <x:c r="E5" s="222"/>
       <x:c r="H5" s="227" t="str">
-        <x:v>What the stronger design changes</x:v>
+        <x:v>Panel model results</x:v>
       </x:c>
       <x:c r="I5" s="227"/>
       <x:c r="J5" s="227"/>
@@ -6889,10 +6889,10 @@
         <x:v>Complaints per 100k</x:v>
       </x:c>
       <x:c r="H6" s="246" t="str">
-        <x:v>1. Between-state result: richer states consistently report higher losses. The pooled income elasticity for loss per capita is 1.55 (p &lt; 0.001).
+        <x:v>1. Between-state result: richer states tend to report higher losses. The pooled income elasticity for loss per capita is 1.55 (p &lt; 0.001).
 2. Within-state result: after state and year fixed effects, income is positive but imprecise (2.19; p = 0.28). Four years provide limited within-state variation.
 3. Robustness: excluding D.C. leaves a positive income elasticity of 0.89 (p &lt; 0.001); winsorizing tails gives 1.18 (p &lt; 0.001).
-4. Conclusion: the evidence supports a robust geographic association, not a causal claim that income growth produces fraud losses.</x:v>
+4. Conclusion: the evidence supports a geographic association, not a causal claim that income growth produces reported losses.</x:v>
       </x:c>
       <x:c r="I6" s="247"/>
       <x:c r="J6" s="247"/>
@@ -7308,7 +7308,7 @@
     <x:mergeCell ref="A35:N38"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2499f5b385946bb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R420231db72b54285"/>
 </x:worksheet>
 </file>
 
@@ -10412,7 +10412,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6820dcbb3cf147bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac51b197c0af4b72"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20688,7 +20688,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cee8195a76a4f5e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9be00b39dd6b403e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21105,7 +21105,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc19f8e4bfe84828"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92a9b18c421f46de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>